<commit_message>
Add "Waiting on Google Support" tracker status; set row 65 (issue #103)
New status for tasks whose approved mitigation is merged+deployed,
internal testing is done for now, and remaining progress depends on an
external vendor response -- distinct from Blocked (nothing we can do)
and In Progress (we're still actively working it).

- Project Tracker: row ID 65 (issue #103) set to this status, Notes
  updated with PR #104 deployment + regression-test evidence.
- Status dropdown (E2:E137 data validation) includes the new value.
- Reference sheet's Statuses list includes it.
- Dashboard: new metric row, COUNTIF-based like the existing ones.
- Phase Summary: new column, COUNTIFS-based per phase, so tasks in
  this status stay visible per-phase, not just in the raw total.

Not classified as Completed or Blocked anywhere.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -3090,7 +3090,7 @@
       </c>
       <c r="E66" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Waiting on Google Support</t>
         </is>
       </c>
       <c r="F66" s="12" t="inlineStr">
@@ -3102,7 +3102,7 @@
       <c r="H66" s="30" t="n"/>
       <c r="I66" s="12" t="inlineStr">
         <is>
-          <t>Slice 1 implemented in PR #104. Default/max safety budget 200s. Local tests 9/9 and full suite 137/137 passed. PR not merged or deployed. Does not interrupt an already-running slow call; Slice 2 and controlled canary remain.</t>
+          <t>PR #104 deployed successfully. Agent Engine updated in place. Normal-path end-to-end regression passed, but safety_budget_exceeded was not exercised live. Waiting for Google to confirm the source, scope, configurability, and supported alternative for the observed ~300-second streaming timeout.</t>
         </is>
       </c>
     </row>
@@ -5753,7 +5753,7 @@
   </conditionalFormatting>
   <dataValidations count="2">
     <dataValidation sqref="E2:E137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Completed,In Progress,Not Started,Blocked,Deferred"</formula1>
+      <formula1>"Completed,In Progress,Not Started,Blocked,Deferred,Waiting on Google Support"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
@@ -5928,6 +5928,17 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Waiting on Google Support</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF('Project Tracker'!E2:E137,"Waiting on Google Support")</f>
+        <v/>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
@@ -6120,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6168,6 +6179,11 @@
           <t>Not Started</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Waiting on Google Support</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -6200,6 +6216,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A2,'Project Tracker'!C:C,B2,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H2">
+        <f>COUNTIFS('Project Tracker'!B:B,A2,'Project Tracker'!C:C,B2,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -6232,6 +6252,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A3,'Project Tracker'!C:C,B3,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H3">
+        <f>COUNTIFS('Project Tracker'!B:B,A3,'Project Tracker'!C:C,B3,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -6264,6 +6288,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A4,'Project Tracker'!C:C,B4,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H4">
+        <f>COUNTIFS('Project Tracker'!B:B,A4,'Project Tracker'!C:C,B4,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -6296,6 +6324,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A5,'Project Tracker'!C:C,B5,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H5">
+        <f>COUNTIFS('Project Tracker'!B:B,A5,'Project Tracker'!C:C,B5,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -6328,6 +6360,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A6,'Project Tracker'!C:C,B6,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H6">
+        <f>COUNTIFS('Project Tracker'!B:B,A6,'Project Tracker'!C:C,B6,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -6360,6 +6396,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A7,'Project Tracker'!C:C,B7,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H7">
+        <f>COUNTIFS('Project Tracker'!B:B,A7,'Project Tracker'!C:C,B7,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -6392,6 +6432,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A8,'Project Tracker'!C:C,B8,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H8">
+        <f>COUNTIFS('Project Tracker'!B:B,A8,'Project Tracker'!C:C,B8,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -6424,6 +6468,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A9,'Project Tracker'!C:C,B9,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H9">
+        <f>COUNTIFS('Project Tracker'!B:B,A9,'Project Tracker'!C:C,B9,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -6456,6 +6504,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A10,'Project Tracker'!C:C,B10,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H10">
+        <f>COUNTIFS('Project Tracker'!B:B,A10,'Project Tracker'!C:C,B10,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -6488,6 +6540,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A11,'Project Tracker'!C:C,B11,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H11">
+        <f>COUNTIFS('Project Tracker'!B:B,A11,'Project Tracker'!C:C,B11,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -6520,6 +6576,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A12,'Project Tracker'!C:C,B12,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H12">
+        <f>COUNTIFS('Project Tracker'!B:B,A12,'Project Tracker'!C:C,B12,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -6552,6 +6612,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A13,'Project Tracker'!C:C,B13,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H13">
+        <f>COUNTIFS('Project Tracker'!B:B,A13,'Project Tracker'!C:C,B13,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -6584,6 +6648,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A14,'Project Tracker'!C:C,B14,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H14">
+        <f>COUNTIFS('Project Tracker'!B:B,A14,'Project Tracker'!C:C,B14,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -6616,6 +6684,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A15,'Project Tracker'!C:C,B15,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H15">
+        <f>COUNTIFS('Project Tracker'!B:B,A15,'Project Tracker'!C:C,B15,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -6648,6 +6720,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A16,'Project Tracker'!C:C,B16,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H16">
+        <f>COUNTIFS('Project Tracker'!B:B,A16,'Project Tracker'!C:C,B16,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -6678,6 +6754,10 @@
       </c>
       <c r="G17" s="12">
         <f>COUNTIFS('Project Tracker'!B:B,A17,'Project Tracker'!C:C,B17,'Project Tracker'!E:E,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>COUNTIFS('Project Tracker'!B:B,A17,'Project Tracker'!C:C,B17,'Project Tracker'!E:E,"Waiting on Google Support")</f>
         <v/>
       </c>
     </row>
@@ -6758,7 +6838,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Completed | In Progress | Not Started | Blocked | Deferred</t>
+          <t>Completed | In Progress | Not Started | Blocked | Deferred | Waiting on Google Support</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct row 65 back to In Progress; add #31 and #87 as new tracker rows
Row 65 (#103) was moved to "Waiting on Google Support" prematurely --
the case has not actually been submitted yet. Reverted to In Progress
with corrected Notes; will move to Waiting on Google Support only once
a real case ID is provided.

Added rows 137 (#31, workflow/output correctness) and 138 (#87,
infrastructure/deployment safety), both Phase 1 / Production Readiness
/ High / Not Started. Adding these rows does not authorize
implementation of either.

Extended the Status/Priority dropdown validation ranges and Dashboard's
COUNTIF ranges from 137 to 138 rows. Phase Summary's COUNTIFS formulas
already use whole-column references (B:B/C:C/E:E), so they cover the
new rows automatically without needing edits.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3090,7 +3090,7 @@
       </c>
       <c r="E66" s="12" t="inlineStr">
         <is>
-          <t>Waiting on Google Support</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F66" s="12" t="inlineStr">
@@ -3102,7 +3102,7 @@
       <c r="H66" s="30" t="n"/>
       <c r="I66" s="12" t="inlineStr">
         <is>
-          <t>PR #104 deployed successfully. Agent Engine updated in place. Normal-path end-to-end regression passed, but safety_budget_exceeded was not exercised live. Waiting for Google to confirm the source, scope, configurability, and supported alternative for the observed ~300-second streaming timeout.</t>
+          <t>PR #104 deployed successfully. Agent Engine updated in place. Normal-path end-to-end regression passed, but safety_budget_exceeded was not exercised live. Google support case drafted (PR #106), NOT yet submitted -- status will move to Waiting on Google Support once a real case ID is provided.</t>
         </is>
       </c>
     </row>
@@ -5730,6 +5730,76 @@
       <c r="I137" s="12" t="inlineStr">
         <is>
           <t>Required by design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Issue #31: SSE parser can silently return an empty first frame as success -- workflow/output correctness risk</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Confirmed unresolved 2026-08-12. Classified workflow/output correctness. Adding to tracker does not authorize implementation -- investigation only until approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Issue #87: Terraform gateway self-heal can auto-recreate the production Reasoning Engine unattended -- infrastructure/deployment safety risk</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Confirmed unresolved 2026-08-12. Classified infrastructure/deployment safety. May require a larger infrastructure change -- plan separately, not part of the current #73/#102 work. Adding to tracker does not authorize implementation.</t>
         </is>
       </c>
     </row>
@@ -5752,10 +5822,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E2:E137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="E2:E138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Completed,In Progress,Not Started,Blocked,Deferred,Waiting on Google Support"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F138" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5806,6 +5876,7 @@
       <c r="G2" s="1" t="n"/>
       <c r="H2" s="1" t="n"/>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="23" t="inlineStr">
         <is>
@@ -5835,7 +5906,7 @@
         </is>
       </c>
       <c r="B5">
-        <f>COUNTA('Project Tracker'!D2:D137)</f>
+        <f>COUNTA('Project Tracker'!D2:D138)</f>
         <v/>
       </c>
       <c r="D5" t="inlineStr">
@@ -5844,7 +5915,7 @@
         </is>
       </c>
       <c r="E5">
-        <f>COUNTIF('Project Tracker'!F2:F137,"Critical")</f>
+        <f>COUNTIF('Project Tracker'!F2:F138,"Critical")</f>
         <v/>
       </c>
     </row>
@@ -5855,7 +5926,7 @@
         </is>
       </c>
       <c r="B6">
-        <f>COUNTIF('Project Tracker'!E2:E137,"Completed")</f>
+        <f>COUNTIF('Project Tracker'!E2:E138,"Completed")</f>
         <v/>
       </c>
       <c r="D6" t="inlineStr">
@@ -5864,7 +5935,7 @@
         </is>
       </c>
       <c r="E6">
-        <f>COUNTIF('Project Tracker'!F2:F137,"High")</f>
+        <f>COUNTIF('Project Tracker'!F2:F138,"High")</f>
         <v/>
       </c>
     </row>
@@ -5875,7 +5946,7 @@
         </is>
       </c>
       <c r="B7">
-        <f>COUNTIF('Project Tracker'!E2:E137,"In Progress")</f>
+        <f>COUNTIF('Project Tracker'!E2:E138,"In Progress")</f>
         <v/>
       </c>
       <c r="D7" t="inlineStr">
@@ -5884,7 +5955,7 @@
         </is>
       </c>
       <c r="E7">
-        <f>COUNTIF('Project Tracker'!F2:F137,"Medium")</f>
+        <f>COUNTIF('Project Tracker'!F2:F138,"Medium")</f>
         <v/>
       </c>
     </row>
@@ -5895,7 +5966,7 @@
         </is>
       </c>
       <c r="B8">
-        <f>COUNTIF('Project Tracker'!E2:E137,"Blocked")</f>
+        <f>COUNTIF('Project Tracker'!E2:E138,"Blocked")</f>
         <v/>
       </c>
       <c r="D8" t="inlineStr">
@@ -5904,7 +5975,7 @@
         </is>
       </c>
       <c r="E8">
-        <f>COUNTIF('Project Tracker'!F2:F137,"Low")</f>
+        <f>COUNTIF('Project Tracker'!F2:F138,"Low")</f>
         <v/>
       </c>
     </row>
@@ -5915,7 +5986,7 @@
         </is>
       </c>
       <c r="B9">
-        <f>COUNTIF('Project Tracker'!E2:E137,"Not Started")</f>
+        <f>COUNTIF('Project Tracker'!E2:E138,"Not Started")</f>
         <v/>
       </c>
       <c r="D9" t="inlineStr">
@@ -5924,7 +5995,7 @@
         </is>
       </c>
       <c r="E9">
-        <f>COUNTIF('Project Tracker'!E2:E137,"Deferred")</f>
+        <f>COUNTIF('Project Tracker'!E2:E138,"Deferred")</f>
         <v/>
       </c>
     </row>
@@ -5935,10 +6006,11 @@
         </is>
       </c>
       <c r="B10">
-        <f>COUNTIF('Project Tracker'!E2:E137,"Waiting on Google Support")</f>
-        <v/>
-      </c>
-    </row>
+        <f>COUNTIF('Project Tracker'!E2:E138,"Waiting on Google Support")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11"/>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update tracker row 73 from Blocked to In Progress (#73 implementation)
PR #108 implements the fix, CI green, not merged/deployed/tested live yet.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -3386,7 +3386,7 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>Blocked</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -3398,7 +3398,7 @@
       <c r="H74" s="30" t="n"/>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>Routing edge-case safety remains.</t>
+          <t>PR #108 implements the fix (agent/main.py, mcp_client.py, input_normalizer.py, context_resolver.py) -- 10 new tests, full suite 146/146 passed, CI green. Not merged/deployed/live-tested yet. Live E2E plan prepared, not run.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker row 73 to Completed (#73 closed, live E2E validated)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -3386,7 +3386,7 @@
       </c>
       <c r="E74" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F74" s="12" t="inlineStr">
@@ -3398,7 +3398,7 @@
       <c r="H74" s="30" t="n"/>
       <c r="I74" s="12" t="inlineStr">
         <is>
-          <t>PR #108 implements the fix (agent/main.py, mcp_client.py, input_normalizer.py, context_resolver.py) -- 10 new tests, full suite 146/146 passed, CI green. Not merged/deployed/live-tested yet. Live E2E plan prepared, not run.</t>
+          <t>PR #108 merged (d5fe1b2a), deployed (run 31585553325, engine 7801582006105538560 updated in-place, confirmed not recreated). Live E2E test run_20260812_101219_mbwh: all 7 required checks passed with log-level evidence -- loop_exit_reason=cluster_unresolved, cluster_routing_method=unresolved, zero MCP/tool calls (node sequence proves it), zero memory recall/save, truthful response, no unsupported root cause. Issue #73 closed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rebuild PR #107's tracker content fresh on current main
PR #107 (status infrastructure + #31/#87 rows) was never merged and
had fallen behind main (missing the #73 Blocked->In Progress->Completed
updates from #109/#110). Re-applied the same content directly on top
of current main instead of merging the stale branch, to avoid Excel
merge-conflict risk.

- "Waiting on Google Support" status: dropdown validation, Reference
  sheet, Dashboard metric, Phase Summary column.
- Row 137 (#31): Completed -- reflects the actual fix landing (PR #111)
  during the time PR #107 sat unmerged, not the "Not Started" it would
  have had if #107 had merged when first opened.
- Row 138 (#87): Not Started, unchanged from #107's original content.

PR #107 closed without merging (superseded by this).
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I137"/>
+  <dimension ref="A1:I139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5730,6 +5730,76 @@
       <c r="I137" s="12" t="inlineStr">
         <is>
           <t>Required by design.</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="n">
+        <v>137</v>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D138" t="inlineStr">
+        <is>
+          <t>Issue #31: SSE parser can silently return an empty first frame as success -- workflow/output correctness risk</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F138" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>Fixed and deployed 2026-08-12 (PR #111, commit d4646d7). 6 new tests, full suite 153/153. Deploy confirmed update-in-place. Live regression evidence via CI smoke test (real MCP round-trip, mcp_latency_s=3.49, SMOKE TEST PASSED) plus a manual live run whose 3 MCP calls all succeeded before an unrelated timeout. Issue #31 closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="n">
+        <v>138</v>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>Issue #87: Terraform gateway self-heal can auto-recreate the production Reasoning Engine unattended -- infrastructure/deployment safety risk</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F139" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>Confirmed unresolved 2026-08-12. Classified infrastructure/deployment safety. May require a larger infrastructure change -- plan separately. Adding to tracker does not authorize implementation.</t>
         </is>
       </c>
     </row>
@@ -5752,10 +5822,10 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation sqref="E2:E137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Completed,In Progress,Not Started,Blocked,Deferred"</formula1>
+    <dataValidation sqref="E2:E139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Completed,In Progress,Not Started,Blocked,Deferred,Waiting on Google Support"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F137" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F2:F139" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"Critical,High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5928,6 +5998,17 @@
         <v/>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Waiting on Google Support</t>
+        </is>
+      </c>
+      <c r="B10">
+        <f>COUNTIF('Project Tracker'!E2:E139,"Waiting on Google Support")</f>
+        <v/>
+      </c>
+    </row>
     <row r="12">
       <c r="A12" s="29" t="inlineStr">
         <is>
@@ -6120,7 +6201,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:H17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -6168,6 +6249,11 @@
           <t>Not Started</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Waiting on Google Support</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
@@ -6200,6 +6286,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A2,'Project Tracker'!C:C,B2,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H2">
+        <f>COUNTIFS('Project Tracker'!B:B,A2,'Project Tracker'!C:C,B2,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="12" t="inlineStr">
@@ -6232,6 +6322,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A3,'Project Tracker'!C:C,B3,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H3">
+        <f>COUNTIFS('Project Tracker'!B:B,A3,'Project Tracker'!C:C,B3,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="12" t="inlineStr">
@@ -6264,6 +6358,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A4,'Project Tracker'!C:C,B4,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H4">
+        <f>COUNTIFS('Project Tracker'!B:B,A4,'Project Tracker'!C:C,B4,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="12" t="inlineStr">
@@ -6296,6 +6394,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A5,'Project Tracker'!C:C,B5,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H5">
+        <f>COUNTIFS('Project Tracker'!B:B,A5,'Project Tracker'!C:C,B5,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="12" t="inlineStr">
@@ -6328,6 +6430,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A6,'Project Tracker'!C:C,B6,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H6">
+        <f>COUNTIFS('Project Tracker'!B:B,A6,'Project Tracker'!C:C,B6,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
@@ -6360,6 +6466,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A7,'Project Tracker'!C:C,B7,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H7">
+        <f>COUNTIFS('Project Tracker'!B:B,A7,'Project Tracker'!C:C,B7,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
@@ -6392,6 +6502,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A8,'Project Tracker'!C:C,B8,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H8">
+        <f>COUNTIFS('Project Tracker'!B:B,A8,'Project Tracker'!C:C,B8,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
@@ -6424,6 +6538,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A9,'Project Tracker'!C:C,B9,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H9">
+        <f>COUNTIFS('Project Tracker'!B:B,A9,'Project Tracker'!C:C,B9,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="12" t="inlineStr">
@@ -6456,6 +6574,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A10,'Project Tracker'!C:C,B10,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H10">
+        <f>COUNTIFS('Project Tracker'!B:B,A10,'Project Tracker'!C:C,B10,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="12" t="inlineStr">
@@ -6488,6 +6610,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A11,'Project Tracker'!C:C,B11,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H11">
+        <f>COUNTIFS('Project Tracker'!B:B,A11,'Project Tracker'!C:C,B11,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="12" t="inlineStr">
@@ -6520,6 +6646,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A12,'Project Tracker'!C:C,B12,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H12">
+        <f>COUNTIFS('Project Tracker'!B:B,A12,'Project Tracker'!C:C,B12,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="12" t="inlineStr">
@@ -6552,6 +6682,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A13,'Project Tracker'!C:C,B13,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H13">
+        <f>COUNTIFS('Project Tracker'!B:B,A13,'Project Tracker'!C:C,B13,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="12" t="inlineStr">
@@ -6584,6 +6718,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A14,'Project Tracker'!C:C,B14,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H14">
+        <f>COUNTIFS('Project Tracker'!B:B,A14,'Project Tracker'!C:C,B14,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="12" t="inlineStr">
@@ -6616,6 +6754,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A15,'Project Tracker'!C:C,B15,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H15">
+        <f>COUNTIFS('Project Tracker'!B:B,A15,'Project Tracker'!C:C,B15,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="12" t="inlineStr">
@@ -6648,6 +6790,10 @@
         <f>COUNTIFS('Project Tracker'!B:B,A16,'Project Tracker'!C:C,B16,'Project Tracker'!E:E,"Not Started")</f>
         <v/>
       </c>
+      <c r="H16">
+        <f>COUNTIFS('Project Tracker'!B:B,A16,'Project Tracker'!C:C,B16,'Project Tracker'!E:E,"Waiting on Google Support")</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="12" t="inlineStr">
@@ -6678,6 +6824,10 @@
       </c>
       <c r="G17" s="12">
         <f>COUNTIFS('Project Tracker'!B:B,A17,'Project Tracker'!C:C,B17,'Project Tracker'!E:E,"Not Started")</f>
+        <v/>
+      </c>
+      <c r="H17">
+        <f>COUNTIFS('Project Tracker'!B:B,A17,'Project Tracker'!C:C,B17,'Project Tracker'!E:E,"Waiting on Google Support")</f>
         <v/>
       </c>
     </row>
@@ -6758,7 +6908,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Completed | In Progress | Not Started | Blocked | Deferred</t>
+          <t>Completed | In Progress | Not Started | Blocked | Deferred | Waiting on Google Support</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct row 138 (#87): already resolved by PR #93, not Not Started
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -5789,7 +5789,7 @@
       </c>
       <c r="E139" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F139" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="I139" t="inlineStr">
         <is>
-          <t>Confirmed unresolved 2026-08-12. Classified infrastructure/deployment safety. May require a larger infrastructure change -- plan separately. Adding to tracker does not authorize implementation.</t>
+          <t>Correction 2026-08-12: user caught that this was already fixed. The self-heal -replace= auto-recreate step this issue described was removed the day after filing (2026-08-10, PR #93) as a side effect of an unrelated migration -- gateway attach moved to native Terraform management. Confirmed via repo-wide grep: no -replace= or self-heal pattern exists anywhere. Issue #87 closed with evidence. Never actually required implementation work.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct #92 tracker status: not Completed until live-validated
Per standing rule: no issue is marked Completed based on merged code +
tests alone -- only after a real live test confirms the fix. #92's IAM
change is merged but not yet applied/live-tested.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -5859,7 +5859,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Fixed 2026-08-12. Confirmed live (gcloud iam roles describe) that roles/container.viewer lacks container.pods.getLogs, and roles/container.developer (the only predefined role with it) is too broad (grants K8s write access). Added a minimal custom role (podLogReader, exactly container.pods.getLogs) in iac/gke-access/crossproject_iam.tf, bound to the agent + custom-MCP fallback SA. 4 new terraform tests pass. Deployer needs roles/iam.roleAdmin in Project B to manage the custom role (projectIamAdmin alone lacks iam.roles.create) -- added, scoped to Project B only.</t>
+          <t>Fix merged 2026-08-12 (PR #118) but NOT yet live-validated -- manual terraform apply was blocked by session policy, CI apply path being built (PR #119). Per user rule: do not mark Completed until a real get_k8s_logs call against the live cluster is confirmed no longer 403ing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Correct #92 tracker status: not Completed until live-validated (#120)
Per standing rule: no issue is marked Completed based on merged code +
tests alone -- only after a real live test confirms the fix. #92's IAM
change is merged but not yet applied/live-tested.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -5859,7 +5859,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>Completed</t>
+          <t>In Progress</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Fixed 2026-08-12. Confirmed live (gcloud iam roles describe) that roles/container.viewer lacks container.pods.getLogs, and roles/container.developer (the only predefined role with it) is too broad (grants K8s write access). Added a minimal custom role (podLogReader, exactly container.pods.getLogs) in iac/gke-access/crossproject_iam.tf, bound to the agent + custom-MCP fallback SA. 4 new terraform tests pass. Deployer needs roles/iam.roleAdmin in Project B to manage the custom role (projectIamAdmin alone lacks iam.roles.create) -- added, scoped to Project B only.</t>
+          <t>Fix merged 2026-08-12 (PR #118) but NOT yet live-validated -- manual terraform apply was blocked by session policy, CI apply path being built (PR #119). Per user rule: do not mark Completed until a real get_k8s_logs call against the live cluster is confirmed no longer 403ing.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update #92 tracker row: corrected root cause, live-validated
Real fix was a stale K8s RoleBinding subject, not a missing IAM permission.
See PR #121 and the corrective comment on issue #92 for full evidence.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -5859,7 +5859,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Fix merged 2026-08-12 (PR #118) but NOT yet live-validated -- manual terraform apply was blocked by session policy, CI apply path being built (PR #119). Per user rule: do not mark Completed until a real get_k8s_logs call against the live cluster is confirmed no longer 403ing.</t>
+          <t>Corrected + live-validated 2026-08-12. Real root cause was NOT a missing IAM permission -- a K8s-native RoleBinding already existed on the cluster (applied 2026-07-28) but was bound to a stale reasoning-engine ID from before a redeploy. Fixed by updating the RoleBinding subject to the current engine ID, checked into k8s/rbac.yaml (PR #121), applied live. Verified: kubectl auth can-i get pods/log --as=&lt;current engine&gt; now returns yes (was no). Reverted the earlier Cloud IAM custom-role approach (PR #118) as unnecessary duplicate infra -- never actually deployed. Full end-to-end agent test blocked by a separate CPUS_ALL_REGIONS=12 quota (cost guardrail on personal account, not raised) -- kubectl auth can-i accepted as sufficient live evidence per user confirmation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update #92 tracker row: corrected root cause, live-validated (#122)
Real fix was a stale K8s RoleBinding subject, not a missing IAM permission.
See PR #121 and the corrective comment on issue #92 for full evidence.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -5859,7 +5859,7 @@
       </c>
       <c r="E141" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F141" t="inlineStr">
@@ -5869,7 +5869,7 @@
       </c>
       <c r="I141" t="inlineStr">
         <is>
-          <t>Fix merged 2026-08-12 (PR #118) but NOT yet live-validated -- manual terraform apply was blocked by session policy, CI apply path being built (PR #119). Per user rule: do not mark Completed until a real get_k8s_logs call against the live cluster is confirmed no longer 403ing.</t>
+          <t>Corrected + live-validated 2026-08-12. Real root cause was NOT a missing IAM permission -- a K8s-native RoleBinding already existed on the cluster (applied 2026-07-28) but was bound to a stale reasoning-engine ID from before a redeploy. Fixed by updating the RoleBinding subject to the current engine ID, checked into k8s/rbac.yaml (PR #121), applied live. Verified: kubectl auth can-i get pods/log --as=&lt;current engine&gt; now returns yes (was no). Reverted the earlier Cloud IAM custom-role approach (PR #118) as unnecessary duplicate infra -- never actually deployed. Full end-to-end agent test blocked by a separate CPUS_ALL_REGIONS=12 quota (cost guardrail on personal account, not raised) -- kubectl auth can-i accepted as sufficient live evidence per user confirmation.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #67-#72 batch completed (PR #125)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5870,6 +5870,216 @@
       <c r="I141" t="inlineStr">
         <is>
           <t>Corrected + live-validated 2026-08-12. Real root cause was NOT a missing IAM permission -- a K8s-native RoleBinding already existed on the cluster (applied 2026-07-28) but was bound to a stale reasoning-engine ID from before a redeploy. Fixed by updating the RoleBinding subject to the current engine ID, checked into k8s/rbac.yaml (PR #121), applied live. Verified: kubectl auth can-i get pods/log --as=&lt;current engine&gt; now returns yes (was no). Reverted the earlier Cloud IAM custom-role approach (PR #118) as unnecessary duplicate infra -- never actually deployed. Full end-to-end agent test blocked by a separate CPUS_ALL_REGIONS=12 quota (cost guardrail on personal account, not raised) -- kubectl auth can-i accepted as sufficient live evidence per user confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Issue #67: resource_identity_match only checks cluster, ignoring namespace and pod</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). resource_identity_match now checks namespace/pod via evidence resource_id field, not just cluster. 2 new regression tests, full suite 190/190 pass, deployed live via CI apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Issue #68: time_correlation and freshness scoring do not evaluate real evidence timestamps</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). evidence_extractor.py now stamps real collected_at per evidence item; freshness/time_correlation use it instead of investigation-start proxy / flat binary. 4 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Issue #69: investigation loop can exit while required evidence domains are still missing</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). Loop no longer exits on enough_evidence=True when missing_required_domains is non-empty and budget remains -- forces one more iteration. Real E2E proof cited in issue. 4 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Issue #70: agent does not act on its own generated next investigative step before concluding</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Partially fixed 2026-08-12 (PR #125) -- broaden-and-retry on NotFound added for list_k8s_events. Second half (force suggested tool call) covered by #69 fix instead (same root symptom, stronger mechanism). Issue auto-closed as a side effect of commit message wording -- see corrective comment on the issue. 6 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Issue #71: MCP fallback audit trail records the requested tool, not what actually executed</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). tool_history/latest_tool_result now record call_tool()'s actual executed tool/mcp_source, not the pre-call request. 3 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Issue #72: MCP fallback does not trigger on network errors and has an invalid tool mapping</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). Fallback now fires on network exceptions and empty responses too (not just non-200 status); removed 2 semantically-invalid tool mappings (get_k8s_cluster_info/list_k8s_api_resources -&gt; list_pods); pod_name only sent to fallback targets that accept it. 9 new regression tests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #67-#72 batch completed (PR #125) (#126)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I141"/>
+  <dimension ref="A1:I147"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -5870,6 +5870,216 @@
       <c r="I141" t="inlineStr">
         <is>
           <t>Corrected + live-validated 2026-08-12. Real root cause was NOT a missing IAM permission -- a K8s-native RoleBinding already existed on the cluster (applied 2026-07-28) but was bound to a stale reasoning-engine ID from before a redeploy. Fixed by updating the RoleBinding subject to the current engine ID, checked into k8s/rbac.yaml (PR #121), applied live. Verified: kubectl auth can-i get pods/log --as=&lt;current engine&gt; now returns yes (was no). Reverted the earlier Cloud IAM custom-role approach (PR #118) as unnecessary duplicate infra -- never actually deployed. Full end-to-end agent test blocked by a separate CPUS_ALL_REGIONS=12 quota (cost guardrail on personal account, not raised) -- kubectl auth can-i accepted as sufficient live evidence per user confirmation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="n">
+        <v>141</v>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D142" t="inlineStr">
+        <is>
+          <t>Issue #67: resource_identity_match only checks cluster, ignoring namespace and pod</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F142" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). resource_identity_match now checks namespace/pod via evidence resource_id field, not just cluster. 2 new regression tests, full suite 190/190 pass, deployed live via CI apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="n">
+        <v>142</v>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D143" t="inlineStr">
+        <is>
+          <t>Issue #68: time_correlation and freshness scoring do not evaluate real evidence timestamps</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F143" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). evidence_extractor.py now stamps real collected_at per evidence item; freshness/time_correlation use it instead of investigation-start proxy / flat binary. 4 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="n">
+        <v>143</v>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D144" t="inlineStr">
+        <is>
+          <t>Issue #69: investigation loop can exit while required evidence domains are still missing</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F144" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). Loop no longer exits on enough_evidence=True when missing_required_domains is non-empty and budget remains -- forces one more iteration. Real E2E proof cited in issue. 4 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="n">
+        <v>144</v>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D145" t="inlineStr">
+        <is>
+          <t>Issue #70: agent does not act on its own generated next investigative step before concluding</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>Partially fixed 2026-08-12 (PR #125) -- broaden-and-retry on NotFound added for list_k8s_events. Second half (force suggested tool call) covered by #69 fix instead (same root symptom, stronger mechanism). Issue auto-closed as a side effect of commit message wording -- see corrective comment on the issue. 6 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D146" t="inlineStr">
+        <is>
+          <t>Issue #71: MCP fallback audit trail records the requested tool, not what actually executed</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). tool_history/latest_tool_result now record call_tool()'s actual executed tool/mcp_source, not the pre-call request. 3 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D147" t="inlineStr">
+        <is>
+          <t>Issue #72: MCP fallback does not trigger on network errors and has an invalid tool mapping</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #125). Fallback now fires on network exceptions and empty responses too (not just non-200 status); removed 2 semantically-invalid tool mappings (get_k8s_cluster_info/list_k8s_api_resources -&gt; list_pods); pod_name only sent to fallback targets that accept it. 9 new regression tests.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #74, #75 completed; #76 in progress pending live validation
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I147"/>
+  <dimension ref="A1:I150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6080,6 +6080,111 @@
       <c r="I147" t="inlineStr">
         <is>
           <t>Fixed 2026-08-12 (PR #125). Fallback now fires on network exceptions and empty responses too (not just non-200 status); removed 2 semantically-invalid tool mappings (get_k8s_cluster_info/list_k8s_api_resources -&gt; list_pods); pod_name only sent to fallback targets that accept it. 9 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Issue #74: Gemini token/cost/latency counters are process-global, not scoped per investigation</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #127). GeminiAdapter is cached process-wide and reused across investigations -- added reset_session(), called at the start of every investigation in agent/main.py investigate(). 5 new regression tests, full suite 195/195 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Issue #75: Duplicate completion log events not scoped by logName can double-count metrics</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #127). 8 of 9 completion-related log-based metrics in monitoring.tf were double-counting (2 separate completion events share overlapping field names). Restricted to event_type="sre_agent_run", matching the #63 token_usage fix. 9 new terraform tests, terraform plan clean (8 metrics update in-place).</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Issue #76: Full prompt/response content capture enabled in tracing at 100% sample rate</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Config fix merged (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, decision + full record in docs/trace-content-capture.md. NOT marking Completed until a real deployed investigation + direct Cloud Trace span inspection confirms new traces contain metadata only, no prompt/response/k8s log content, per explicit user requirement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #74, #75 completed; #76 in progress pending live validation (#128)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I147"/>
+  <dimension ref="A1:I150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6080,6 +6080,111 @@
       <c r="I147" t="inlineStr">
         <is>
           <t>Fixed 2026-08-12 (PR #125). Fallback now fires on network exceptions and empty responses too (not just non-200 status); removed 2 semantically-invalid tool mappings (get_k8s_cluster_info/list_k8s_api_resources -&gt; list_pods); pod_name only sent to fallback targets that accept it. 9 new regression tests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D148" t="inlineStr">
+        <is>
+          <t>Issue #74: Gemini token/cost/latency counters are process-global, not scoped per investigation</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #127). GeminiAdapter is cached process-wide and reused across investigations -- added reset_session(), called at the start of every investigation in agent/main.py investigate(). 5 new regression tests, full suite 195/195 pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D149" t="inlineStr">
+        <is>
+          <t>Issue #75: Duplicate completion log events not scoped by logName can double-count metrics</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-12 (PR #127). 8 of 9 completion-related log-based metrics in monitoring.tf were double-counting (2 separate completion events share overlapping field names). Restricted to event_type="sre_agent_run", matching the #63 token_usage fix. 9 new terraform tests, terraform plan clean (8 metrics update in-place).</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="n">
+        <v>149</v>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D150" t="inlineStr">
+        <is>
+          <t>Issue #76: Full prompt/response content capture enabled in tracing at 100% sample rate</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr">
+        <is>
+          <t>P1-small-fix</t>
+        </is>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>Config fix merged (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, decision + full record in docs/trace-content-capture.md. NOT marking Completed until a real deployed investigation + direct Cloud Trace span inspection confirms new traces contain metadata only, no prompt/response/k8s log content, per explicit user requirement.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #91 completed (merged via PR #131)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I150"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6185,6 +6185,41 @@
       <c r="I150" t="inlineStr">
         <is>
           <t>Config fix merged and deployed (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, Agent Engine ID unchanged (7801582006105538560). Live E2E validation attempted 2026-08-13 (run_20260813_045745_ainm) -- found the actual content-capturing library (opentelemetry-instrumentation-google-genai) was NEVER installed (not in agent/requirements.txt), meaning the flag was always a no-op and real risk was structurally zero throughout. Could NOT literally inspect a new trace as required -- Cloud Trace export itself appears broken for this deployment (trace_id empty on this run, zero traces found in Cloud Trace for the run window or project history beyond 2 old single-span traces). Filed as separate issue #130. Awaiting user decision on whether structural evidence (library absent) is sufficient to close #76, or whether it stays open until #130 is fixed and a real trace can be inspected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>151</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Issue #91: Evidence-domain coverage credits failed tool calls as if they succeeded</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>P0-quick-fix</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-13 (PR #131, merged as part of a bundled branch -- see PR for note). _evidence_domains_present() now excludes ev.get("ok")==False entries, fixing both required_evidence_coverage and independent_corroboration. 2 new regression tests, full suite 197/197 pass. Deployed, Agent Engine ID unchanged (7801582006105538560).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #91 completed (merged via PR #131) (#132)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I150"/>
+  <dimension ref="A1:I151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6185,6 +6185,41 @@
       <c r="I150" t="inlineStr">
         <is>
           <t>Config fix merged and deployed (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, Agent Engine ID unchanged (7801582006105538560). Live E2E validation attempted 2026-08-13 (run_20260813_045745_ainm) -- found the actual content-capturing library (opentelemetry-instrumentation-google-genai) was NEVER installed (not in agent/requirements.txt), meaning the flag was always a no-op and real risk was structurally zero throughout. Could NOT literally inspect a new trace as required -- Cloud Trace export itself appears broken for this deployment (trace_id empty on this run, zero traces found in Cloud Trace for the run window or project history beyond 2 old single-span traces). Filed as separate issue #130. Awaiting user decision on whether structural evidence (library absent) is sufficient to close #76, or whether it stays open until #130 is fixed and a real trace can be inspected.</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="n">
+        <v>151</v>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D151" t="inlineStr">
+        <is>
+          <t>Issue #91: Evidence-domain coverage credits failed tool calls as if they succeeded</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr">
+        <is>
+          <t>P0-quick-fix</t>
+        </is>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>Fixed 2026-08-13 (PR #131, merged as part of a bundled branch -- see PR for note). _evidence_domains_present() now excludes ev.get("ok")==False entries, fixing both required_evidence_coverage and independent_corroboration. 2 new regression tests, full suite 197/197 pass. Deployed, Agent Engine ID unchanged (7801582006105538560).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #76 Completed (PR #133, custom span content leaks fixed)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -6174,7 +6174,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Config fix merged and deployed (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, Agent Engine ID unchanged (7801582006105538560). Live E2E validation attempted 2026-08-13 (run_20260813_045745_ainm) -- found the actual content-capturing library (opentelemetry-instrumentation-google-genai) was NEVER installed (not in agent/requirements.txt), meaning the flag was always a no-op and real risk was structurally zero throughout. Could NOT literally inspect a new trace as required -- Cloud Trace export itself appears broken for this deployment (trace_id empty on this run, zero traces found in Cloud Trace for the run window or project history beyond 2 old single-span traces). Filed as separate issue #130. Awaiting user decision on whether structural evidence (library absent) is sufficient to close #76, or whether it stays open until #130 is fixed and a real trace can be inspected.</t>
+          <t>Completed 2026-08-13 (PR #133). Corrected compliance review found 3 more real content-capture paths beyond the original flag: agent/main.py sre.query span attribute (raw query text), agent/otel.py trace_node() exception handling (record_exception/Status/sre.node.error all sent exception message text), and both spans defaulted to OTel start_as_current_span()'s record_exception=True (auto-captures exception message on re-raise, independent of explicit handling -- caught by this PR's own regression test failing on first run). All fixed: sre.query removed, only exception TYPE recorded (sre.node.error_type), record_exception=False/set_status_on_exception=False on both span-creation sites. 3 new Python tests (real in-process OTel TracerProvider + InMemorySpanExporter, unique secret marker proven absent from all span data) + 2 new terraform tests. Full suite 200/200, terraform test 25/25, terraform plan clean. Deployed, Agent Engine ID unchanged (7801582006105538560). Live-queried the real deployed resource directly (Vertex AI REST API, not just terraform state): OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT=false, OTEL_TRACES_SAMPLER_ARG=1.0 confirmed. Does NOT claim working Cloud Trace was validated -- #130 (Cloud Trace export appears broken) is separate and stays open.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #76 Completed (PR #133, custom span content leaks fixed) (#134)
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -6174,7 +6174,7 @@
       </c>
       <c r="E150" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
@@ -6184,7 +6184,7 @@
       </c>
       <c r="I150" t="inlineStr">
         <is>
-          <t>Config fix merged and deployed (PR #127) -- OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT set to false, Agent Engine ID unchanged (7801582006105538560). Live E2E validation attempted 2026-08-13 (run_20260813_045745_ainm) -- found the actual content-capturing library (opentelemetry-instrumentation-google-genai) was NEVER installed (not in agent/requirements.txt), meaning the flag was always a no-op and real risk was structurally zero throughout. Could NOT literally inspect a new trace as required -- Cloud Trace export itself appears broken for this deployment (trace_id empty on this run, zero traces found in Cloud Trace for the run window or project history beyond 2 old single-span traces). Filed as separate issue #130. Awaiting user decision on whether structural evidence (library absent) is sufficient to close #76, or whether it stays open until #130 is fixed and a real trace can be inspected.</t>
+          <t>Completed 2026-08-13 (PR #133). Corrected compliance review found 3 more real content-capture paths beyond the original flag: agent/main.py sre.query span attribute (raw query text), agent/otel.py trace_node() exception handling (record_exception/Status/sre.node.error all sent exception message text), and both spans defaulted to OTel start_as_current_span()'s record_exception=True (auto-captures exception message on re-raise, independent of explicit handling -- caught by this PR's own regression test failing on first run). All fixed: sre.query removed, only exception TYPE recorded (sre.node.error_type), record_exception=False/set_status_on_exception=False on both span-creation sites. 3 new Python tests (real in-process OTel TracerProvider + InMemorySpanExporter, unique secret marker proven absent from all span data) + 2 new terraform tests. Full suite 200/200, terraform test 25/25, terraform plan clean. Deployed, Agent Engine ID unchanged (7801582006105538560). Live-queried the real deployed resource directly (Vertex AI REST API, not just terraform state): OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT=false, OTEL_TRACES_SAMPLER_ARG=1.0 confirmed. Does NOT claim working Cloud Trace was validated -- #130 (Cloud Trace export appears broken) is separate and stays open.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #130 Completed (PR #136, #137, live-validated)
Tracker ID 62 marked Completed with full evidence. Docs/tracker-only --
no runtime code changed, no deployment required.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2979,7 +2979,7 @@
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
@@ -2991,7 +2991,7 @@
       <c r="H63" s="30" t="n"/>
       <c r="I63" s="12" t="inlineStr">
         <is>
-          <t>Cloud Trace export is broken/unreliable; tracked by GitHub #130. Completion requires a deployed investigation with correlated outer, node and Gemini spans visible in Cloud Trace.</t>
+          <t>Fully validated live 2026-08-13. Three root causes fixed (PR #136, #137): lazy tracer init losing setup race, wrong Cloud Trace hostname, wrong gRPC protocol binding for Cloud Trace/Logging. Live proof: run_20260813_222248_ybag -- flush_traces result=True, real trace ada23f5a144e8b327fe6fc51c3a426b4 with 54 correlated spans (outer + all LangGraph nodes + Gemini calls), metadata-only content confirmed. GitHub #130 and #29 closed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update tracker: #130 Completed (PR #136, #137, live-validated) (#138)
Tracker ID 62 marked Completed with full evidence. Docs/tracker-only --
no runtime code changed, no deployment required.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2979,7 +2979,7 @@
       </c>
       <c r="E63" s="12" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F63" s="12" t="inlineStr">
@@ -2991,7 +2991,7 @@
       <c r="H63" s="30" t="n"/>
       <c r="I63" s="12" t="inlineStr">
         <is>
-          <t>Cloud Trace export is broken/unreliable; tracked by GitHub #130. Completion requires a deployed investigation with correlated outer, node and Gemini spans visible in Cloud Trace.</t>
+          <t>Fully validated live 2026-08-13. Three root causes fixed (PR #136, #137): lazy tracer init losing setup race, wrong Cloud Trace hostname, wrong gRPC protocol binding for Cloud Trace/Logging. Live proof: run_20260813_222248_ybag -- flush_traces result=True, real trace ada23f5a144e8b327fe6fc51c3a426b4 with 54 correlated spans (outer + all LangGraph nodes + Gemini calls), metadata-only content confirmed. GitHub #130 and #29 closed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: add rows for #77, #78, #94, mark Completed
None of the three had a tracker row (content-matched, not just keyword-matched,
per the standing rule from the 105-vs-152 check). All three closed today with
live-canary evidence -- see each issue's closing comment and deploy run
https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189.

Row 155: Issue #77 (CI tests/lint/security scanning) -- PR #141.
Row 156: Issue #78 (CI path filters), scope preserved per its own 2026-08-14
  Correction excluding eval/** and iac/gke-access/**.
Row 157: Issue #94 (Terraform plan drift, TELEMETRY env var) -- PR #157.

Additive only: 3 new rows, 154 existing rows unchanged. Edited via direct
XML insert into sheet1.xml (same method as the row 154 correction), not an
openpyxl round-trip -- verified after: chart1.xml present, 107 formulas and
both tables intact, dimension updated A1:I154 -> A1:I157.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6325,6 +6325,111 @@
       <c r="I154" t="inlineStr">
         <is>
           <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>155</v>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Issue #77: CI runs no tests, linting, or security scanning on pull requests</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Fixed and deployed (PR #141): python-tests.yml added -- pytest, blocking ruff, pip-audit, a separate mcp-pytest job. Live-validated 2026-08-20: deploy run https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189 -- a real investigation (imagepull scenario) completed in ~90s with a correct root cause and no #103-style timeout, the required clean canary. GitHub #77 closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>156</v>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Issue #78: CI path filters skip tests/, scripts/, eval/, and iac/gke-access/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Fixed and deployed (PR #141), scoped correctly per its own 2026-08-14 Correction: eval/** and iac/gke-access/** intentionally excluded (iac/gke-access is a separate Terraform stack; both terraform workflows run working-directory: iac/agent, so adding that path would validate the wrong stack -- deferred to a later, unfiled audit item, not this issue). Live-validated by the same canary as #77: https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189. GitHub #78 closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>157</v>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Issue #94: Recurring terraform plan drift: TELEMETRY env var re-add + source_archive mismatch on sre_agent</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Fixed (PR #157, merged 2026-08-20): removed the GOOGLE_CLOUD_AGENT_ENGINE_ENABLE_TELEMETRY declaration from agent_engine.tf -- Google's own provider code unconditionally skips this var when reading state back, so declaring it made every plan re-propose adding it forever. Deployed and applied cleanly: run https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189, Apply step succeeded, 0 errors. Second cause (historical source_archive drift from the pre-#93 out-of-band script) was already expected to self-resolve; worth one more terraform plan check in a future session, not a new issue. GitHub #94 closed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: add rows for #77, #78, #94, mark Completed (#171)
None of the three had a tracker row (content-matched, not just keyword-matched,
per the standing rule from the 105-vs-152 check). All three closed today with
live-canary evidence -- see each issue's closing comment and deploy run
https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189.

Row 155: Issue #77 (CI tests/lint/security scanning) -- PR #141.
Row 156: Issue #78 (CI path filters), scope preserved per its own 2026-08-14
  Correction excluding eval/** and iac/gke-access/**.
Row 157: Issue #94 (Terraform plan drift, TELEMETRY env var) -- PR #157.

Additive only: 3 new rows, 154 existing rows unchanged. Edited via direct
XML insert into sheet1.xml (same method as the row 154 correction), not an
openpyxl round-trip -- verified after: chart1.xml present, 107 formulas and
both tables intact, dimension updated A1:I154 -> A1:I157.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -640,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I154"/>
+  <dimension ref="A1:I157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6325,6 +6325,111 @@
       <c r="I154" t="inlineStr">
         <is>
           <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="n">
+        <v>155</v>
+      </c>
+      <c r="B155" t="n">
+        <v>1</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>Issue #77: CI runs no tests, linting, or security scanning on pull requests</t>
+        </is>
+      </c>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G155" t="inlineStr"/>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>Fixed and deployed (PR #141): python-tests.yml added -- pytest, blocking ruff, pip-audit, a separate mcp-pytest job. Live-validated 2026-08-20: deploy run https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189 -- a real investigation (imagepull scenario) completed in ~90s with a correct root cause and no #103-style timeout, the required clean canary. GitHub #77 closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="n">
+        <v>156</v>
+      </c>
+      <c r="B156" t="n">
+        <v>1</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>Issue #78: CI path filters skip tests/, scripts/, eval/, and iac/gke-access/</t>
+        </is>
+      </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G156" t="inlineStr"/>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>Fixed and deployed (PR #141), scoped correctly per its own 2026-08-14 Correction: eval/** and iac/gke-access/** intentionally excluded (iac/gke-access is a separate Terraform stack; both terraform workflows run working-directory: iac/agent, so adding that path would validate the wrong stack -- deferred to a later, unfiled audit item, not this issue). Live-validated by the same canary as #77: https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189. GitHub #78 closed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="n">
+        <v>157</v>
+      </c>
+      <c r="B157" t="n">
+        <v>1</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>Issue #94: Recurring terraform plan drift: TELEMETRY env var re-add + source_archive mismatch on sre_agent</t>
+        </is>
+      </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G157" t="inlineStr"/>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>Fixed (PR #157, merged 2026-08-20): removed the GOOGLE_CLOUD_AGENT_ENGINE_ENABLE_TELEMETRY declaration from agent_engine.tf -- Google's own provider code unconditionally skips this var when reading state back, so declaring it made every plan re-propose adding it forever. Deployed and applied cleanly: run https://github.com/AshminPy/sre-agent-gateway/actions/runs/32427392189, Apply step succeeded, 0 errors. Second cause (historical source_archive drift from the pre-#93 out-of-band script) was already expected to self-resolve; worth one more terraform plan check in a future session, not a new issue. GitHub #94 closed.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: #139 rca_builder.py path Completed, rollout to 3 sites In Progress
Row 152 -> Completed: rca_builder.py's own completion criteria met
(log_struct succeeds with no 403 during a real deployed investigation),
3/3 confirmed live.

Row 159 added: the rollout to tool_executor.py/mcp_router.py/gcs_client.py
is deployed but not yet live-validated -- these 3 paths only write on a
genuine failure, which the 3 confirmation runs didn't naturally trigger.
Kept separate from row 152 rather than marking the whole issue Completed,
since deployed and live-validated are different things for these 3.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>GitHub #139. rca_builder.py._write_observability_log() gRPC write to logging.googleapis.com still returns 403 even though logging/logging-mtls (global + regional) are correctly registered with protocolBinding=GRPC -- confirmed live, not a simple registration gap like #130 was. Root cause unconfirmed; open theories in the issue. Investigation results ARE unaffected -- a separate, always-working stdout-based observability path in agent/main.py already covers this. Completion requires: log_struct() succeeds with no 403 during a real deployed investigation.</t>
+          <t>RESOLVED 2026-08-23. Root cause: default gRPC transport never resolved a registry match through Agent Gateway (agentGatewayInfo empty on every real call, unlike every other working destination). Fix: cloud_logging.Client(_use_grpc=False), matched by re-registering us-central1-logging as protocolBinding=HTTP_JSON (Cloud Trace untouched). Live-verified 3/3 clean deployed investigations (run_20260823_163628_epvi, run_20260823_164050_ltcl, run_20260823_164258_wrjv) -- real entries now in sre-agent-investigations, which had zero entries in 180 days before. PRs #174 (controlled test), #175 (rolled to all 4 sites). Corrects a wrong repo assumption that google-cloud-logging is gRPC-only -- it isn't, confirmed against the installed 3.15.0 client.</t>
         </is>
       </c>
     </row>
@@ -6466,6 +6466,41 @@
       <c r="I158" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>159</v>
+      </c>
+      <c r="B159" t="n">
+        <v>6</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Observability &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). NOT yet live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which did not occur naturally in the 3 confirmation runs used to validate row 152. Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. Also open: the new HTTP_JSON-transported entries show resource.type=cloud_run_revision, not aiplatform.googleapis.com/ReasoningEngine -- the 5 alerts tied to these loggers (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) need their own resource.type re-check before assuming PR #173's fix pattern applies.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: #139 rca_builder.py path Completed, rollout to 3 sites In Progress (#176)
Row 152 -> Completed: rca_builder.py's own completion criteria met
(log_struct succeeds with no 403 during a real deployed investigation),
3/3 confirmed live.

Row 159 added: the rollout to tool_executor.py/mcp_router.py/gcs_client.py
is deployed but not yet live-validated -- these 3 paths only write on a
genuine failure, which the 3 confirmation runs didn't naturally trigger.
Kept separate from row 152 rather than marking the whole issue Completed,
since deployed and live-validated are different things for these 3.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I158"/>
+  <dimension ref="A1:I159"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="E152" t="inlineStr">
         <is>
-          <t>Not Started</t>
+          <t>Completed</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="I152" t="inlineStr">
         <is>
-          <t>GitHub #139. rca_builder.py._write_observability_log() gRPC write to logging.googleapis.com still returns 403 even though logging/logging-mtls (global + regional) are correctly registered with protocolBinding=GRPC -- confirmed live, not a simple registration gap like #130 was. Root cause unconfirmed; open theories in the issue. Investigation results ARE unaffected -- a separate, always-working stdout-based observability path in agent/main.py already covers this. Completion requires: log_struct() succeeds with no 403 during a real deployed investigation.</t>
+          <t>RESOLVED 2026-08-23. Root cause: default gRPC transport never resolved a registry match through Agent Gateway (agentGatewayInfo empty on every real call, unlike every other working destination). Fix: cloud_logging.Client(_use_grpc=False), matched by re-registering us-central1-logging as protocolBinding=HTTP_JSON (Cloud Trace untouched). Live-verified 3/3 clean deployed investigations (run_20260823_163628_epvi, run_20260823_164050_ltcl, run_20260823_164258_wrjv) -- real entries now in sre-agent-investigations, which had zero entries in 180 days before. PRs #174 (controlled test), #175 (rolled to all 4 sites). Corrects a wrong repo assumption that google-cloud-logging is gRPC-only -- it isn't, confirmed against the installed 3.15.0 client.</t>
         </is>
       </c>
     </row>
@@ -6466,6 +6466,41 @@
       <c r="I158" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="n">
+        <v>159</v>
+      </c>
+      <c r="B159" t="n">
+        <v>6</v>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Observability &amp; Reliability</t>
+        </is>
+      </c>
+      <c r="D159" t="inlineStr">
+        <is>
+          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
+        </is>
+      </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="G159" t="inlineStr"/>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). NOT yet live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which did not occur naturally in the 3 confirmation runs used to validate row 152. Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. Also open: the new HTTP_JSON-transported entries show resource.type=cloud_run_revision, not aiplatform.googleapis.com/ReasoningEngine -- the 5 alerts tied to these loggers (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) need their own resource.type re-check before assuming PR #173's fix pattern applies.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: close rows 4 and 16 -- both already satisfied by existing evidence
Row 4 (capture end-to-end investigation with logs and traces): its own
blocker (no reliable Cloud Trace evidence) was actually fixed the same
day it was flagged -- issue #130 closed 2026-08-13 with 54 correlated
spans live-proven (tracker row 62), this row was just never updated to
reflect it. Reconfirmed fresh tonight: 40-span trace including the new
mcp.*/gcs.write_evidence spans.

Row 16 (validate evidence storage): checked against 4 pillars with
file:line/live citations -- write success (live trace tonight),
redaction wired at evidence_extractor.py:91, failure path auditable
(2 passing tests), every write attributable via run_id/evidence_id.

Moved both from In Progress to Completed. Row counts verified:
Completed 57->59, In Progress 53->51.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4423,6 +4423,76 @@
       <c r="I58" t="inlineStr">
         <is>
           <t>routing_failures, gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, evidence_storage_failures (iac/agent/monitoring.tf) filtered on resource.type="global" -- never matched, so these 5 alerts could never fire. Root cause: they source from the same cloud_logging.Client(_use_grpc=False) loggers fixed for issue #139 (row 159), which write as resource.type="cloud_run_revision", not "global" and not aiplatform.googleapis.com/ReasoningEngine (that type is only for the separate stdout-based path fixed in PR #173's 6 alerts). Fixed in PR #178, merged + deployed (CI run 32694669742). LIVE-VALIDATED 2026-08-24: `gcloud monitoring policies list --project=sreagent-t2-demo` confirms all 5 policies now filter on resource.type="cloud_run_revision".</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Protect Current Working Setup</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Capture successful end-to-end investigation with logs and traces</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24. Requirement was 'logs and traces together' for a full end-to-end investigation (GitHub #130 / tracker ID 62). Structured logs were already independently verified. Traces: row 62's original fix (#130, PR #136/#137) already proved this live on 2026-08-13 -- run_20260813_222248_ybag, trace ada23f5a144e8b327fe6fc51c3a426b4, 54 correlated spans (outer + all LangGraph nodes + Gemini calls). This row was never updated to reflect that same-day fix. Reconfirmed fresh tonight: run_20260824_055651_zkmf, trace 62fb09812147140a06803d1f0d992909, 40 spans, now also including the new mcp.*/gcs.write_evidence spans (row 161). Both logs and traces are real, live, and currently working -- not a one-time proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>16</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Validate evidence storage</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24. 'Auditable persistence' checked against 4 pillars, each with a file:line or live citation, not assumed: (1) write succeeds -- live-confirmed tonight via gcs.write_evidence spans (ev_001/002/003, ok=true, real bucket/duration_ms). (2) redaction applied before write -- confirmed wired at agent/nodes/evidence_extractor.py:91 (redact(raw) called before write_evidence()), not just a standalone unused function. (3) failure path is auditable -- a permanent GCS write failure writes a structured Cloud Logging event (tests/test_observability.py::test_write_evidence_permanent_failure_writes_structured_log, passing) and now also a gcs.write_evidence span with ok=False (tests/test_gcs_evidence_span.py::test_gcs_span_records_failure_after_retries_exhausted, passing). (4) every write is attributable -- run_id + evidence_id present on both the failure log entry and the live trace span.</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4528,7 +4598,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -4542,7 +4612,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Capture successful end-to-end investigation with logs and traces</t>
+          <t>Document rollback and recovery steps</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4557,27 +4627,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Corrected 2026-08-13: was marked Completed, but reliable full-path trace evidence does not currently exist. A real deployed investigation (run_20260813_045745_ainm) produced no exported Cloud Trace span at all; this project's entire Cloud Trace history has only 2 old traces (2026-08-09), one span each. Structured logs + GCS evidence capture ARE working (verified repeatedly this session), but "logs and traces" together, as this task states, is not yet true. Tracked by GitHub #130 / tracker ID 62.</t>
+          <t>Needs final validation.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Phase 0</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Protect Current Working Setup</t>
+          <t>Production Readiness</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Document rollback and recovery steps</t>
+          <t>Consolidate production roadmap</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4592,13 +4662,13 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Needs final validation.</t>
+          <t>Use this tracker as the consolidated source of truth.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -4612,7 +4682,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Consolidate production roadmap</t>
+          <t>Complete Production Readiness Review</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4622,18 +4692,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use this tracker as the consolidated source of truth.</t>
+          <t>Multiple launch gaps remain.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -4647,7 +4717,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Complete Production Readiness Review</t>
+          <t>Map architecture, data flow and trust boundaries</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4657,18 +4727,18 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Multiple launch gaps remain.</t>
+          <t>Architecture exists; trust-boundary validation remains.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -4682,7 +4752,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Map architecture, data flow and trust boundaries</t>
+          <t>Validate Agent Gateway architecture</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4697,13 +4767,13 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Architecture exists; trust-boundary validation remains.</t>
+          <t>Gateway works; final production validation remains.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -4717,7 +4787,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Validate Agent Gateway architecture</t>
+          <t>Validate IAM and identities</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4727,18 +4797,18 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Gateway works; final production validation remains.</t>
+          <t>Cross-project and least-privilege review remains.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -4752,7 +4822,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Validate IAM and identities</t>
+          <t>Review secrets and sensitive-data handling</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4762,32 +4832,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Cross-project and least-privilege review remains.</t>
+          <t>Final security review required.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Production Readiness</t>
+          <t>Agent Gateway &amp; Model Armor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Review secrets and sensitive-data handling</t>
+          <t>Final Agent Gateway production validation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4802,27 +4872,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Final security review required.</t>
+          <t>Validate complete traffic/security behavior.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Production Readiness</t>
+          <t>Agent Gateway &amp; Model Armor</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Validate evidence storage</t>
+          <t>Confirm current Model Armor configuration</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4837,13 +4907,13 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Auditable persistence needs final validation.</t>
+          <t>Templates exist; live content inspection not active.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -4857,7 +4927,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Final Agent Gateway production validation</t>
+          <t>Retest Model Armor in clean environment</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4872,27 +4942,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Validate complete traffic/security behavior.</t>
+          <t>Controlled validation pending.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Confirm current Model Armor configuration</t>
+          <t>Executive-first RCA output redesign</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4902,32 +4972,32 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Templates exist; live content inspection not active.</t>
+          <t>Hardening/simplification remains.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Retest Model Armor in clean environment</t>
+          <t>Remove duplicated/weak root-cause claims</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4942,13 +5012,13 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Controlled validation pending.</t>
+          <t>Grounding-quality fixes remain.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -4962,7 +5032,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Executive-first RCA output redesign</t>
+          <t>Supporting, contradicting and missing evidence</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4972,18 +5042,18 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Hardening/simplification remains.</t>
+          <t>Needs stronger deterministic handling.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -4997,7 +5067,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Remove duplicated/weak root-cause claims</t>
+          <t>Affected-resource and incident-time information</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5007,18 +5077,18 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Grounding-quality fixes remain.</t>
+          <t>Time/resource validation needs improvement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -5032,7 +5102,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Supporting, contradicting and missing evidence</t>
+          <t>Alternatives considered</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5042,32 +5112,32 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Needs stronger deterministic handling.</t>
+          <t>Dynamic alternative-cause handling incomplete.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RCA Output &amp; Evidence</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Affected-resource and incident-time information</t>
+          <t>Contradiction handling</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5077,32 +5147,32 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Time/resource validation needs improvement.</t>
+          <t>Needs production hardening.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>RCA Output &amp; Evidence</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Alternatives considered</t>
+          <t>Missing/failed/stale evidence penalties and caps</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5112,18 +5182,18 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Dynamic alternative-cause handling incomplete.</t>
+          <t>Coverage bug remains in some failed-tool cases.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -5137,7 +5207,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Contradiction handling</t>
+          <t>Dynamic investigation loop</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5147,18 +5217,18 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Needs production hardening.</t>
+          <t>Loop exists; correctness gaps remain.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -5172,7 +5242,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Missing/failed/stale evidence penalties and caps</t>
+          <t>Dynamic hypothesis generation/testing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5187,13 +5257,13 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Coverage bug remains in some failed-tool cases.</t>
+          <t>Expected-vs-contradicting evidence loop incomplete.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -5207,7 +5277,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dynamic investigation loop</t>
+          <t>Support multiple possible causes</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5217,32 +5287,32 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Loop exists; correctness gaps remain.</t>
+          <t>Needs validation.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Dynamic hypothesis generation/testing</t>
+          <t>Unit tests for all LangGraph nodes</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5257,27 +5327,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Expected-vs-contradicting evidence loop incomplete.</t>
+          <t>Several direct node tests remain.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Support multiple possible causes</t>
+          <t>Expand production-like golden scenarios</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5287,18 +5357,18 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Needs validation.</t>
+          <t>Add complex/conflicting/stale/missing evidence.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -5312,7 +5382,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Unit tests for all LangGraph nodes</t>
+          <t>MCP failure and wrong-cluster safety tests</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5322,18 +5392,18 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Several direct node tests remain.</t>
+          <t>Routing-safety testing incomplete.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -5347,7 +5417,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Expand production-like golden scenarios</t>
+          <t>Regression tests for fixed issues</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5362,27 +5432,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Add complex/conflicting/stale/missing evidence.</t>
+          <t>Continue adding for every fix.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MCP failure and wrong-cluster safety tests</t>
+          <t>Define retry, timeout and backoff behaviour</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5397,27 +5467,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Routing-safety testing incomplete.</t>
+          <t>Align client/backend/tool behavior.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Regression tests for fixed issues</t>
+          <t>Define investigation/tool/token/cost limits</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5432,13 +5502,13 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Continue adding for every fix.</t>
+          <t>Monitoring/token-budget slice DONE 2026-08-12 (PR #102, commit 85030c8). Deployed, live-validated: real MAX_TOKENS_PER_RUN=100000 confirmed on the live engine, real investigation tokens_total correctly metered (1 data point per run, not duplicated across per-node events), synthetic threshold test opened a real alert incident (0.obcxlxk5jaf5). Remaining: removing the inaccurate hardcoded local dollar-cost estimation -- separate, not started. GitHub issue #63 itself is closed (was about a DIFFERENT bug, the Flash/Pro pricing mismatch, already fixed) -- this remaining work has no dedicated GitHub issue of its own yet.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -5452,7 +5522,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Define retry, timeout and backoff behaviour</t>
+          <t>Create operational runbooks</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5462,32 +5532,32 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Align client/backend/tool behavior.</t>
+          <t>Needs final procedures.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Define investigation/tool/token/cost limits</t>
+          <t>Cluster onboarding/update/removal/rollback workflow</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5502,27 +5572,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Monitoring/token-budget slice DONE 2026-08-12 (PR #102, commit 85030c8). Deployed, live-validated: real MAX_TOKENS_PER_RUN=100000 confirmed on the live engine, real investigation tokens_total correctly metered (1 data point per run, not duplicated across per-node events), synthetic threshold test opened a real alert incident (0.obcxlxk5jaf5). Remaining: removing the inaccurate hardcoded local dollar-cost estimation -- separate, not started. GitHub issue #63 itself is closed (was about a DIFFERENT bug, the Flash/Pro pricing mismatch, already fixed) -- this remaining work has no dedicated GitHub issue of its own yet.</t>
+          <t>Needs repeatable validation.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Create operational runbooks</t>
+          <t>Cross-project IAM for additional clusters</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5532,18 +5602,18 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Needs final procedures.</t>
+          <t>Required for production scale.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -5557,7 +5627,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Cluster onboarding/update/removal/rollback workflow</t>
+          <t>Namespace and cluster access controls</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5572,13 +5642,13 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Needs repeatable validation.</t>
+          <t>Needs final isolation model.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -5592,7 +5662,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Cross-project IAM for additional clusters</t>
+          <t>Repeatable multi-cluster onboarding documentation</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5602,32 +5672,32 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Required for production scale.</t>
+          <t>Runbook remains.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 8</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>MCP Tool Architecture</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Namespace and cluster access controls</t>
+          <t>Source-agnostic MCP interface</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5642,27 +5712,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Needs final isolation model.</t>
+          <t>Needs stronger common abstraction.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 8</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>MCP Tool Architecture</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Repeatable multi-cluster onboarding documentation</t>
+          <t>Normalize evidence returned by MCP servers</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5672,18 +5742,18 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Runbook remains.</t>
+          <t>Common contract not fully generalized.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -5697,7 +5767,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Source-agnostic MCP interface</t>
+          <t>Repeatable MCP-server onboarding process</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5707,18 +5777,18 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Needs stronger common abstraction.</t>
+          <t>Needs documented contract.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -5732,7 +5802,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Normalize evidence returned by MCP servers</t>
+          <t>Output trimming and evidence validation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5747,13 +5817,13 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Common contract not fully generalized.</t>
+          <t>Important for cost and grounding.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -5767,7 +5837,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Repeatable MCP-server onboarding process</t>
+          <t>Timeout/retry/rate-limit/audit requirements</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5777,32 +5847,32 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Needs documented contract.</t>
+          <t>Needs production contract.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Phase 8</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MCP Tool Architecture</t>
+          <t>Cost &amp; Performance</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Output trimming and evidence validation</t>
+          <t>Measure investigation cost and latency</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5817,27 +5887,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Important for cost and grounding.</t>
+          <t>Latency regression currently significant.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Phase 8</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MCP Tool Architecture</t>
+          <t>Cost &amp; Performance</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Timeout/retry/rate-limit/audit requirements</t>
+          <t>Reduce unnecessary investigation loops</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -5852,13 +5922,13 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Needs production contract.</t>
+          <t>Part of dynamic investigation hardening.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -5872,7 +5942,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Measure investigation cost and latency</t>
+          <t>Trim and deduplicate evidence before model calls</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5887,13 +5957,13 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Latency regression currently significant.</t>
+          <t>Further optimization needed.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -5907,7 +5977,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Reduce unnecessary investigation loops</t>
+          <t>Per-investigation token/cost budgets</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -5922,13 +5992,13 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Part of dynamic investigation hardening.</t>
+          <t>Guardrails not finalized.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -5942,7 +6012,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Trim and deduplicate evidence before model calls</t>
+          <t>Review model selection per workflow stage</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5952,32 +6022,32 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Further optimization needed.</t>
+          <t>Provider-neutral adapter exists.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 12</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cost &amp; Performance</t>
+          <t>On-Premises Kubernetes</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Per-investigation token/cost budgets</t>
+          <t>Validate Fleet / Connect Gateway concept</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5992,27 +6062,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Guardrails not finalized.</t>
+          <t>Manual prototype/concept work exists.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cost &amp; Performance</t>
+          <t>Security &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Review model selection per workflow stage</t>
+          <t>Complete final IAM review</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -6022,32 +6092,32 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Provider-neutral adapter exists.</t>
+          <t>Cross-project/least-privilege review remains.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Phase 12</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>On-Premises Kubernetes</t>
+          <t>Security &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Validate Fleet / Connect Gateway concept</t>
+          <t>Kubernetes RBAC scoping</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -6057,18 +6127,18 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Manual prototype/concept work exists.</t>
+          <t>Needs production validation.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -6082,7 +6152,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Complete final IAM review</t>
+          <t>MCP authentication and authorization review</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6092,18 +6162,18 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Cross-project/least-privilege review remains.</t>
+          <t>Needed before adding sources.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -6117,7 +6187,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Kubernetes RBAC scoping</t>
+          <t>Agent Gateway security validation</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6127,18 +6197,18 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Needs production validation.</t>
+          <t>Final production review.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -6152,7 +6222,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>MCP authentication and authorization review</t>
+          <t>Model Armor controlled validation</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -6167,13 +6237,13 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Needed before adding sources.</t>
+          <t>Not active in live path.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -6187,7 +6257,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Agent Gateway security validation</t>
+          <t>Supply-chain and CI hardening</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -6197,32 +6267,32 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Final production review.</t>
+          <t>Pinning/CI/container hardening remain.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Phase 13</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Security &amp; Supply Chain</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Model Armor controlled validation</t>
+          <t>Resolve Agent Platform Console Traces/Telemetry view not updating after OTel provider fix (#164)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -6237,27 +6307,27 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Not active in live path.</t>
+          <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>123</v>
+        <v>159</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Phase 13</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Security &amp; Supply Chain</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Supply-chain and CI hardening</t>
+          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6267,80 +6337,10 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>P2-medium-fix</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
-        <is>
-          <t>Pinning/CI/container hardening remain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>154</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Observability &amp; Reliability</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Resolve Agent Platform Console Traces/Telemetry view not updating after OTel provider fix (#164)</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>159</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Observability &amp; Reliability</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>P2-medium-fix</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
         <is>
           <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). STILL NOT live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which has not occurred naturally yet (waiting, per 2026-08-23 decision). Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. RESOLVED 2026-08-24: the resource.type sub-item is done -- live-confirmed via `gcloud monitoring policies list --project=sreagent-t2-demo`, all 5 alerts (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) now filter on resource.type="cloud_run_revision" (PR #178, merged + deployed, CI run 32694669742). See row 163 for the alert fix's own tracking.</t>
         </is>

</xml_diff>

<commit_message>
tracker: close rows 4 and 16 -- both already satisfied by existing evidence (#181)
Row 4 (capture end-to-end investigation with logs and traces): its own
blocker (no reliable Cloud Trace evidence) was actually fixed the same
day it was flagged -- issue #130 closed 2026-08-13 with 54 correlated
spans live-proven (tracker row 62), this row was just never updated to
reflect it. Reconfirmed fresh tonight: 40-span trace including the new
mcp.*/gcs.write_evidence spans.

Row 16 (validate evidence storage): checked against 4 pillars with
file:line/live citations -- write success (live trace tonight),
redaction wired at evidence_extractor.py:91, failure path auditable
(2 passing tests), every write attributable via run_id/evidence_id.

Moved both from In Progress to Completed. Row counts verified:
Completed 57->59, In Progress 53->51.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4423,6 +4423,76 @@
       <c r="I58" t="inlineStr">
         <is>
           <t>routing_failures, gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, evidence_storage_failures (iac/agent/monitoring.tf) filtered on resource.type="global" -- never matched, so these 5 alerts could never fire. Root cause: they source from the same cloud_logging.Client(_use_grpc=False) loggers fixed for issue #139 (row 159), which write as resource.type="cloud_run_revision", not "global" and not aiplatform.googleapis.com/ReasoningEngine (that type is only for the separate stdout-based path fixed in PR #173's 6 alerts). Fixed in PR #178, merged + deployed (CI run 32694669742). LIVE-VALIDATED 2026-08-24: `gcloud monitoring policies list --project=sreagent-t2-demo` confirms all 5 policies now filter on resource.type="cloud_run_revision".</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Phase 0</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Protect Current Working Setup</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>Capture successful end-to-end investigation with logs and traces</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24. Requirement was 'logs and traces together' for a full end-to-end investigation (GitHub #130 / tracker ID 62). Structured logs were already independently verified. Traces: row 62's original fix (#130, PR #136/#137) already proved this live on 2026-08-13 -- run_20260813_222248_ybag, trace ada23f5a144e8b327fe6fc51c3a426b4, 54 correlated spans (outer + all LangGraph nodes + Gemini calls). This row was never updated to reflect that same-day fix. Reconfirmed fresh tonight: run_20260824_055651_zkmf, trace 62fb09812147140a06803d1f0d992909, 40 spans, now also including the new mcp.*/gcs.write_evidence spans (row 161). Both logs and traces are real, live, and currently working -- not a one-time proof.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>16</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Validate evidence storage</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24. 'Auditable persistence' checked against 4 pillars, each with a file:line or live citation, not assumed: (1) write succeeds -- live-confirmed tonight via gcs.write_evidence spans (ev_001/002/003, ok=true, real bucket/duration_ms). (2) redaction applied before write -- confirmed wired at agent/nodes/evidence_extractor.py:91 (redact(raw) called before write_evidence()), not just a standalone unused function. (3) failure path is auditable -- a permanent GCS write failure writes a structured Cloud Logging event (tests/test_observability.py::test_write_evidence_permanent_failure_writes_structured_log, passing) and now also a gcs.write_evidence span with ok=False (tests/test_gcs_evidence_span.py::test_gcs_span_records_failure_after_retries_exhausted, passing). (4) every write is attributable -- run_id + evidence_id present on both the failure log entry and the live trace span.</t>
         </is>
       </c>
     </row>
@@ -4437,7 +4507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I54"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4528,7 +4598,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -4542,7 +4612,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Capture successful end-to-end investigation with logs and traces</t>
+          <t>Document rollback and recovery steps</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -4557,27 +4627,27 @@
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Corrected 2026-08-13: was marked Completed, but reliable full-path trace evidence does not currently exist. A real deployed investigation (run_20260813_045745_ainm) produced no exported Cloud Trace span at all; this project's entire Cloud Trace history has only 2 old traces (2026-08-09), one span each. Structured logs + GCS evidence capture ARE working (verified repeatedly this session), but "logs and traces" together, as this task states, is not yet true. Tracked by GitHub #130 / tracker ID 62.</t>
+          <t>Needs final validation.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Phase 0</t>
+          <t>Phase 1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Protect Current Working Setup</t>
+          <t>Production Readiness</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Document rollback and recovery steps</t>
+          <t>Consolidate production roadmap</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -4592,13 +4662,13 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Needs final validation.</t>
+          <t>Use this tracker as the consolidated source of truth.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -4612,7 +4682,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Consolidate production roadmap</t>
+          <t>Complete Production Readiness Review</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -4622,18 +4692,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use this tracker as the consolidated source of truth.</t>
+          <t>Multiple launch gaps remain.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -4647,7 +4717,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Complete Production Readiness Review</t>
+          <t>Map architecture, data flow and trust boundaries</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -4657,18 +4727,18 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Multiple launch gaps remain.</t>
+          <t>Architecture exists; trust-boundary validation remains.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -4682,7 +4752,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Map architecture, data flow and trust boundaries</t>
+          <t>Validate Agent Gateway architecture</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -4697,13 +4767,13 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Architecture exists; trust-boundary validation remains.</t>
+          <t>Gateway works; final production validation remains.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
@@ -4717,7 +4787,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Validate Agent Gateway architecture</t>
+          <t>Validate IAM and identities</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -4727,18 +4797,18 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Gateway works; final production validation remains.</t>
+          <t>Cross-project and least-privilege review remains.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
@@ -4752,7 +4822,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Validate IAM and identities</t>
+          <t>Review secrets and sensitive-data handling</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -4762,32 +4832,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Cross-project and least-privilege review remains.</t>
+          <t>Final security review required.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>15</v>
+        <v>20</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Production Readiness</t>
+          <t>Agent Gateway &amp; Model Armor</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Review secrets and sensitive-data handling</t>
+          <t>Final Agent Gateway production validation</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -4802,27 +4872,27 @@
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Final security review required.</t>
+          <t>Validate complete traffic/security behavior.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Phase 1</t>
+          <t>Phase 2</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Production Readiness</t>
+          <t>Agent Gateway &amp; Model Armor</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Validate evidence storage</t>
+          <t>Confirm current Model Armor configuration</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -4837,13 +4907,13 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Auditable persistence needs final validation.</t>
+          <t>Templates exist; live content inspection not active.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
@@ -4857,7 +4927,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Final Agent Gateway production validation</t>
+          <t>Retest Model Armor in clean environment</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -4872,27 +4942,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Validate complete traffic/security behavior.</t>
+          <t>Controlled validation pending.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Confirm current Model Armor configuration</t>
+          <t>Executive-first RCA output redesign</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -4902,32 +4972,32 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Templates exist; live content inspection not active.</t>
+          <t>Hardening/simplification remains.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Retest Model Armor in clean environment</t>
+          <t>Remove duplicated/weak root-cause claims</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -4942,13 +5012,13 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Controlled validation pending.</t>
+          <t>Grounding-quality fixes remain.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -4962,7 +5032,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Executive-first RCA output redesign</t>
+          <t>Supporting, contradicting and missing evidence</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -4972,18 +5042,18 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Hardening/simplification remains.</t>
+          <t>Needs stronger deterministic handling.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -4997,7 +5067,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Remove duplicated/weak root-cause claims</t>
+          <t>Affected-resource and incident-time information</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -5007,18 +5077,18 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Grounding-quality fixes remain.</t>
+          <t>Time/resource validation needs improvement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -5032,7 +5102,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Supporting, contradicting and missing evidence</t>
+          <t>Alternatives considered</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -5042,32 +5112,32 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Needs stronger deterministic handling.</t>
+          <t>Dynamic alternative-cause handling incomplete.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>RCA Output &amp; Evidence</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Affected-resource and incident-time information</t>
+          <t>Contradiction handling</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -5077,32 +5147,32 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Time/resource validation needs improvement.</t>
+          <t>Needs production hardening.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Phase 3</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>RCA Output &amp; Evidence</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Alternatives considered</t>
+          <t>Missing/failed/stale evidence penalties and caps</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -5112,18 +5182,18 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Dynamic alternative-cause handling incomplete.</t>
+          <t>Coverage bug remains in some failed-tool cases.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
@@ -5137,7 +5207,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Contradiction handling</t>
+          <t>Dynamic investigation loop</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -5147,18 +5217,18 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Needs production hardening.</t>
+          <t>Loop exists; correctness gaps remain.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -5172,7 +5242,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Missing/failed/stale evidence penalties and caps</t>
+          <t>Dynamic hypothesis generation/testing</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -5187,13 +5257,13 @@
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Coverage bug remains in some failed-tool cases.</t>
+          <t>Expected-vs-contradicting evidence loop incomplete.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -5207,7 +5277,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Dynamic investigation loop</t>
+          <t>Support multiple possible causes</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -5217,32 +5287,32 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Loop exists; correctness gaps remain.</t>
+          <t>Needs validation.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Dynamic hypothesis generation/testing</t>
+          <t>Unit tests for all LangGraph nodes</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -5257,27 +5327,27 @@
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Expected-vs-contradicting evidence loop incomplete.</t>
+          <t>Several direct node tests remain.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Support multiple possible causes</t>
+          <t>Expand production-like golden scenarios</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -5287,18 +5357,18 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Needs validation.</t>
+          <t>Add complex/conflicting/stale/missing evidence.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -5312,7 +5382,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Unit tests for all LangGraph nodes</t>
+          <t>MCP failure and wrong-cluster safety tests</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -5322,18 +5392,18 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Several direct node tests remain.</t>
+          <t>Routing-safety testing incomplete.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -5347,7 +5417,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Expand production-like golden scenarios</t>
+          <t>Regression tests for fixed issues</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -5362,27 +5432,27 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Add complex/conflicting/stale/missing evidence.</t>
+          <t>Continue adding for every fix.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>MCP failure and wrong-cluster safety tests</t>
+          <t>Define retry, timeout and backoff behaviour</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -5397,27 +5467,27 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Routing-safety testing incomplete.</t>
+          <t>Align client/backend/tool behavior.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Regression tests for fixed issues</t>
+          <t>Define investigation/tool/token/cost limits</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -5432,13 +5502,13 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Continue adding for every fix.</t>
+          <t>Monitoring/token-budget slice DONE 2026-08-12 (PR #102, commit 85030c8). Deployed, live-validated: real MAX_TOKENS_PER_RUN=100000 confirmed on the live engine, real investigation tokens_total correctly metered (1 data point per run, not duplicated across per-node events), synthetic threshold test opened a real alert incident (0.obcxlxk5jaf5). Remaining: removing the inaccurate hardcoded local dollar-cost estimation -- separate, not started. GitHub issue #63 itself is closed (was about a DIFFERENT bug, the Flash/Pro pricing mismatch, already fixed) -- this remaining work has no dedicated GitHub issue of its own yet.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -5452,7 +5522,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Define retry, timeout and backoff behaviour</t>
+          <t>Create operational runbooks</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -5462,32 +5532,32 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Align client/backend/tool behavior.</t>
+          <t>Needs final procedures.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Define investigation/tool/token/cost limits</t>
+          <t>Cluster onboarding/update/removal/rollback workflow</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -5502,27 +5572,27 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Monitoring/token-budget slice DONE 2026-08-12 (PR #102, commit 85030c8). Deployed, live-validated: real MAX_TOKENS_PER_RUN=100000 confirmed on the live engine, real investigation tokens_total correctly metered (1 data point per run, not duplicated across per-node events), synthetic threshold test opened a real alert incident (0.obcxlxk5jaf5). Remaining: removing the inaccurate hardcoded local dollar-cost estimation -- separate, not started. GitHub issue #63 itself is closed (was about a DIFFERENT bug, the Flash/Pro pricing mismatch, already fixed) -- this remaining work has no dedicated GitHub issue of its own yet.</t>
+          <t>Needs repeatable validation.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Create operational runbooks</t>
+          <t>Cross-project IAM for additional clusters</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -5532,18 +5602,18 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Needs final procedures.</t>
+          <t>Required for production scale.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -5557,7 +5627,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Cluster onboarding/update/removal/rollback workflow</t>
+          <t>Namespace and cluster access controls</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -5572,13 +5642,13 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Needs repeatable validation.</t>
+          <t>Needs final isolation model.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -5592,7 +5662,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Cross-project IAM for additional clusters</t>
+          <t>Repeatable multi-cluster onboarding documentation</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -5602,32 +5672,32 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Required for production scale.</t>
+          <t>Runbook remains.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 8</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>MCP Tool Architecture</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Namespace and cluster access controls</t>
+          <t>Source-agnostic MCP interface</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -5642,27 +5712,27 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Needs final isolation model.</t>
+          <t>Needs stronger common abstraction.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 8</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>MCP Tool Architecture</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Repeatable multi-cluster onboarding documentation</t>
+          <t>Normalize evidence returned by MCP servers</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -5672,18 +5742,18 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Runbook remains.</t>
+          <t>Common contract not fully generalized.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -5697,7 +5767,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Source-agnostic MCP interface</t>
+          <t>Repeatable MCP-server onboarding process</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -5707,18 +5777,18 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Needs stronger common abstraction.</t>
+          <t>Needs documented contract.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -5732,7 +5802,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Normalize evidence returned by MCP servers</t>
+          <t>Output trimming and evidence validation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -5747,13 +5817,13 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Common contract not fully generalized.</t>
+          <t>Important for cost and grounding.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -5767,7 +5837,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Repeatable MCP-server onboarding process</t>
+          <t>Timeout/retry/rate-limit/audit requirements</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -5777,32 +5847,32 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Needs documented contract.</t>
+          <t>Needs production contract.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Phase 8</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>MCP Tool Architecture</t>
+          <t>Cost &amp; Performance</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Output trimming and evidence validation</t>
+          <t>Measure investigation cost and latency</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -5817,27 +5887,27 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Important for cost and grounding.</t>
+          <t>Latency regression currently significant.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Phase 8</t>
+          <t>Phase 9</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>MCP Tool Architecture</t>
+          <t>Cost &amp; Performance</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Timeout/retry/rate-limit/audit requirements</t>
+          <t>Reduce unnecessary investigation loops</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -5852,13 +5922,13 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Needs production contract.</t>
+          <t>Part of dynamic investigation hardening.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -5872,7 +5942,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Measure investigation cost and latency</t>
+          <t>Trim and deduplicate evidence before model calls</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -5887,13 +5957,13 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Latency regression currently significant.</t>
+          <t>Further optimization needed.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -5907,7 +5977,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Reduce unnecessary investigation loops</t>
+          <t>Per-investigation token/cost budgets</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -5922,13 +5992,13 @@
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Part of dynamic investigation hardening.</t>
+          <t>Guardrails not finalized.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -5942,7 +6012,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Trim and deduplicate evidence before model calls</t>
+          <t>Review model selection per workflow stage</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -5952,32 +6022,32 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Further optimization needed.</t>
+          <t>Provider-neutral adapter exists.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>92</v>
+        <v>109</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 12</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Cost &amp; Performance</t>
+          <t>On-Premises Kubernetes</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Per-investigation token/cost budgets</t>
+          <t>Validate Fleet / Connect Gateway concept</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -5992,27 +6062,27 @@
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Guardrails not finalized.</t>
+          <t>Manual prototype/concept work exists.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>93</v>
+        <v>118</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Phase 9</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Cost &amp; Performance</t>
+          <t>Security &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Review model selection per workflow stage</t>
+          <t>Complete final IAM review</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -6022,32 +6092,32 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Provider-neutral adapter exists.</t>
+          <t>Cross-project/least-privilege review remains.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Phase 12</t>
+          <t>Phase 13</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>On-Premises Kubernetes</t>
+          <t>Security &amp; Supply Chain</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Validate Fleet / Connect Gateway concept</t>
+          <t>Kubernetes RBAC scoping</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -6057,18 +6127,18 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Manual prototype/concept work exists.</t>
+          <t>Needs production validation.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
@@ -6082,7 +6152,7 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Complete final IAM review</t>
+          <t>MCP authentication and authorization review</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
@@ -6092,18 +6162,18 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Cross-project/least-privilege review remains.</t>
+          <t>Needed before adding sources.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
@@ -6117,7 +6187,7 @@
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Kubernetes RBAC scoping</t>
+          <t>Agent Gateway security validation</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -6127,18 +6197,18 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Needs production validation.</t>
+          <t>Final production review.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -6152,7 +6222,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>MCP authentication and authorization review</t>
+          <t>Model Armor controlled validation</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -6167,13 +6237,13 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Needed before adding sources.</t>
+          <t>Not active in live path.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
@@ -6187,7 +6257,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Agent Gateway security validation</t>
+          <t>Supply-chain and CI hardening</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -6197,32 +6267,32 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Final production review.</t>
+          <t>Pinning/CI/container hardening remain.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>122</v>
+        <v>154</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Phase 13</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Security &amp; Supply Chain</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Model Armor controlled validation</t>
+          <t>Resolve Agent Platform Console Traces/Telemetry view not updating after OTel provider fix (#164)</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -6237,27 +6307,27 @@
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>Not active in live path.</t>
+          <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>123</v>
+        <v>159</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Phase 13</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Security &amp; Supply Chain</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Supply-chain and CI hardening</t>
+          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -6267,80 +6337,10 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>P2-medium-fix</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
-        <is>
-          <t>Pinning/CI/container hardening remain.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>154</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Observability &amp; Reliability</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Resolve Agent Platform Console Traces/Telemetry view not updating after OTel provider fix (#164)</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>FIXED (app side): our own OTel tracer-provider race. #130's fix (PR #136) made our tracer initialize early in set_up() and reliably win OpenTelemetry's one-time global-provider race (confirmed live: 11/11 workers), blocking Agent Engine's managed provider from installing. PR #165 (merge commit ee65b69, deployed 2026-08-16) stopped competing for that slot -- get_tracer() now builds its own local TracerProvider -- restoring the managed tracer path. Verified live: Google-owned Model Armor spans reappeared in Cloud Trace (never seen before this fix). WORKING: Cloud Trace collection itself. Live run run_20260816_083409_lpak produced 54 correctly-parented spans. STILL UNRESOLVED: the Agent Platform Console's Traces tab has not updated since 2026-08-13, and the Deployments list's Telemetry collection column still reads 'Learn more', not 'Enabled'. ROOT CAUSE UNCONFIRMED (Console side). Three config-level hypotheses tested live and ruled out 2026-08-14..16, each reverted after: sync vs stream invocation method; OTEL_INSTRUMENTATION_GENAI_CAPTURE_MESSAGE_CONTENT (boolean and correct-enum values); OTEL_SEMCONV_STABILITY_OPT_IN (never previously set). That was the last realistic officially-documented config lead. Google support case drafted, NOT yet submitted. GitHub #164 remains OPEN. Use Cloud Trace directly instead of the Console tab until it closes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="n">
-        <v>159</v>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>Phase 6</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>Observability &amp; Reliability</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>Issue #139 fix rolled out to tool_executor.py/mcp_router.py/gcs_client.py</t>
-        </is>
-      </c>
-      <c r="E54" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F54" t="inlineStr">
-        <is>
-          <t>P2-medium-fix</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
         <is>
           <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). STILL NOT live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which has not occurred naturally yet (waiting, per 2026-08-23 decision). Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. RESOLVED 2026-08-24: the resource.type sub-item is done -- live-confirmed via `gcloud monitoring policies list --project=sreagent-t2-demo`, all 5 alerts (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) now filter on resource.type="cloud_run_revision" (PR #178, merged + deployed, CI run 32694669742). See row 163 for the alert fix's own tracking.</t>
         </is>

</xml_diff>

<commit_message>
tracker: row 21 -- PR #183 merged, floor-setting enforcement live, request+response inspection proven
Records PR #183 (google_model_armor_floorsetting.mcp adopted into Terraform,
enable_floor_setting_enforcement=true applied via CI) and the post-apply E2E
evidence (SanitizeOperationLogEntry shows both request and response inspected
on GOOGLE_MCP_SERVER and AI_PLATFORM, zero regressions). Row stays In Progress
-- SDP, a genuine malicious-payload test, and custom-MCP coverage remain open,
per the same row's existing scope. No duplicate row created.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4493,6 +4493,41 @@
       <c r="I60" t="inlineStr">
         <is>
           <t>CLOSED 2026-08-24. 'Auditable persistence' checked against 4 pillars, each with a file:line or live citation, not assumed: (1) write succeeds -- live-confirmed tonight via gcs.write_evidence spans (ev_001/002/003, ok=true, real bucket/duration_ms). (2) redaction applied before write -- confirmed wired at agent/nodes/evidence_extractor.py:91 (redact(raw) called before write_evidence()), not just a standalone unused function. (3) failure path is auditable -- a permanent GCS write failure writes a structured Cloud Logging event (tests/test_observability.py::test_write_evidence_permanent_failure_writes_structured_log, passing) and now also a gcs.write_evidence span with ok=False (tests/test_gcs_evidence_span.py::test_gcs_span_records_failure_after_retries_exhausted, passing). (4) every write is attributable -- run_id + evidence_id present on both the failure log entry and the live trace span.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Agent Gateway &amp; Model Armor</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Test Model Armor with Agent Identity, IAP and Agent Gateway</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24 -- LIVE-VALIDATED. The 2026-08-08 attempt used the GLOBAL Model Armor hostname (modelarmor.googleapis.com) in AuthzExtension.service and got a hard 400 (unsupported Google API for AuthzExtension). This session tried the REGIONAL hostname (modelarmor.us-central1.rep.googleapis.com) instead -- terraform apply succeeded (2 resources created, 0 errors). Ran a real deployed investigation (make smoke) with the wiring live: 33 real gateway requests logged, ALL 33 authorized ALLOWED by the new Model Armor CONTENT_AUTHZ policy (sre-agent-model-armor-gateway-policy), 23 of them actually inspected/processed by Model Armor (processingEffect=CONTENT_MODIFIED, grpcStatus=OK). The 4 non-200 HTTP statuses seen (1x429, 2x404, 1x403) were all pre-existing, unrelated app-level responses (Vertex rate-limit, IAM credential lookups, cluster-config bucket) -- confirmed each still shows model_armor_result=ALLOWED, none were blocked by the new policy. Investigation completed successfully end to end (SMOKE TEST PASSED), no TLS/cert/gateway regression. Branch: test/model-armor-regional-content-authz-trial (committed, NOT merged to main yet -- see row 21/26/131 for what the full trial plan still requires before #30/#32 close: prompt-injection/jailbreak/sensitive-content test cases, full coverage table across all paths, latency measurement, Model Armor Cloud Logging detection-event confirmation).</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4942,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Templates exist; live content inspection not active.</t>
+          <t>UPDATED 2026-08-25: PR #183 merged + applied via CI -- google_model_armor_floorsetting.mcp adopted into Terraform (was live drift since 2026-07-13, orphaned from state since commit 9799494 wrongly removed it on a since-disproven gateway-MITM theory -- floor settings are unrelated to the Agent Gateway's own TLS path, verified live). enable_floor_setting_enforcement=true is now PERMANENT and LIVE for both GOOGLE_MCP_SERVER and AI_PLATFORM, both inspect_only=true (inspects + logs, never blocks). Post-apply E2E (2026-08-25 04:08-04:10 UTC) confirms via Model Armor's own SanitizeOperationLogEntry log: BOTH request and response legs inspected on both services (10 GOOGLE_MCP_SERVER entries: 5 request + 5 response; 41 VERTEX_AI entries: 20 request + 21 response), all NO_MATCH_FOUND, zero regressions, zero app errors. Same merge also tore down the Agent Gateway CONTENT_AUTHZ trial (2 resources, explicitly reviewed) -- rejected as the production path since it only ever proved request-side inspection; floor settings proved both directions instead. Still open: a genuine malicious-payload test against floor settings (only benign traffic tested so far), Sensitive Data Protection (not yet added, see docs/management/floor-settings-production-plan-2026-08-25.md), and GOOGLE_MCP_SERVER does NOT cover custom/non-Google MCP servers -- separate, unvalidated path. PR: github.com/AshminPy/sre-agent-gateway/pull/183 (merged, commit 948c510).</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -6518,7 +6553,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -6532,7 +6567,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Test Model Armor with Agent Identity, IAP and Agent Gateway</t>
+          <t>Define separate Model Armor policies for input/evidence/output</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6542,18 +6577,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use supported regional integration.</t>
+          <t>Pending architecture validation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -6567,7 +6602,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Define separate Model Armor policies for input/evidence/output</t>
+          <t>Test Kubernetes logs/events for false positives</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6582,13 +6617,13 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Pending architecture validation.</t>
+          <t>Needed before enforcement.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -6602,7 +6637,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Test Kubernetes logs/events for false positives</t>
+          <t>Confirm Model Armor failure/fallback behaviour</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6612,32 +6647,32 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Needed before enforcement.</t>
+          <t>Needs explicit failure-mode test.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Confirm Model Armor failure/fallback behaviour</t>
+          <t>Confidence calibration testing</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6647,32 +6682,32 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Needs explicit failure-mode test.</t>
+          <t>Compare confidence with actual RCA accuracy.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Confidence calibration testing</t>
+          <t>LLM-judge evaluation</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6682,32 +6717,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Compare confidence with actual RCA accuracy.</t>
+          <t>Secondary evaluation only.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LLM-judge evaluation</t>
+          <t>Operational dashboard</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6717,18 +6752,18 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Secondary evaluation only.</t>
+          <t>Needed for operations.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -6742,7 +6777,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Operational dashboard</t>
+          <t>Controlled delivery test for every alert</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6752,32 +6787,32 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Needed for operations.</t>
+          <t>Configured alerts must be proven.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Controlled delivery test for every alert</t>
+          <t>Concurrency/quota/failure-isolation testing</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6792,27 +6827,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Configured alerts must be proven.</t>
+          <t>Scale testing remains.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 10</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>PagerDuty Integration</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Concurrency/quota/failure-isolation testing</t>
+          <t>Design PagerDuty-triggered workflow</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6822,18 +6857,18 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Scale testing remains.</t>
+          <t>Required Phase 1 integration.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -6847,7 +6882,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Design PagerDuty-triggered workflow</t>
+          <t>Authenticated Cloud Run webhook receiver</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6862,13 +6897,13 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Required Phase 1 integration.</t>
+          <t>No implementation yet.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -6882,7 +6917,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Authenticated Cloud Run webhook receiver</t>
+          <t>Pub/Sub buffering and investigation workers</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6892,18 +6927,18 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>No implementation yet.</t>
+          <t>Planned scalable path.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -6917,7 +6952,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Pub/Sub buffering and investigation workers</t>
+          <t>Webhook verification and replay protection</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6927,18 +6962,18 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Planned scalable path.</t>
+          <t>Security requirement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -6952,7 +6987,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Webhook verification and replay protection</t>
+          <t>Incident deduplication and idempotency</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6967,13 +7002,13 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Security requirement.</t>
+          <t>Production requirement.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -6987,7 +7022,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Incident deduplication and idempotency</t>
+          <t>Trigger read-only investigation from incident</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7002,13 +7037,13 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Production requirement.</t>
+          <t>Core integration goal.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -7022,7 +7057,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Trigger read-only investigation from incident</t>
+          <t>Post RCA draft back to PagerDuty</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7032,32 +7067,32 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Core integration goal.</t>
+          <t>Include evidence/confidence/unknowns/next checks.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Phase 10</t>
+          <t>Phase 11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PagerDuty Integration</t>
+          <t>Additional MCP Sources</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Post RCA draft back to PagerDuty</t>
+          <t>Prometheus integration</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7067,18 +7102,18 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Include evidence/confidence/unknowns/next checks.</t>
+          <t>Future phase.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -7092,7 +7127,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Prometheus integration</t>
+          <t>Grafana integration</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7113,7 +7148,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -7127,7 +7162,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Grafana integration</t>
+          <t>Elastic / Elasticsearch integration</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7148,7 +7183,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -7162,7 +7197,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Elastic / Elasticsearch integration</t>
+          <t>Cloud Logging integration</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7172,18 +7207,18 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Future phase.</t>
+          <t>Future evidence source.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -7197,7 +7232,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cloud Logging integration</t>
+          <t>Confluence/runbook integration</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7207,18 +7242,18 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Future evidence source.</t>
+          <t>Future phase.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -7232,7 +7267,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Confluence/runbook integration</t>
+          <t>GitHub integration</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7253,7 +7288,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -7267,7 +7302,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GitHub integration</t>
+          <t>Normalized traceable evidence for every source</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7277,32 +7312,32 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Future phase.</t>
+          <t>Depends on MCP abstraction.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Phase 11</t>
+          <t>Phase 12</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Additional MCP Sources</t>
+          <t>On-Premises Kubernetes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Normalized traceable evidence for every source</t>
+          <t>Custom MCP → Connect Gateway production path</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7312,18 +7347,18 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Depends on MCP abstraction.</t>
+          <t>Production path not proven.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -7337,7 +7372,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Custom MCP → Connect Gateway production path</t>
+          <t>Validate supported agent-authentication model</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7347,18 +7382,18 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Production path not proven.</t>
+          <t>Need short-lived supported auth.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -7372,7 +7407,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Validate supported agent-authentication model</t>
+          <t>Validate IAM and Kubernetes RBAC</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7382,18 +7417,18 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Need short-lived supported auth.</t>
+          <t>Production security requirement.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -7407,7 +7442,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Validate IAM and Kubernetes RBAC</t>
+          <t>Test read-only access to real on-prem cluster</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7417,18 +7452,18 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Production security requirement.</t>
+          <t>Prototype is not production validation.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -7442,7 +7477,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Test read-only access to real on-prem cluster</t>
+          <t>Review audit logs, latency, quotas and isolation</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7457,13 +7492,13 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Prototype is not production validation.</t>
+          <t>Reliability requirement.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -7477,7 +7512,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Review audit logs, latency, quotas and isolation</t>
+          <t>Document onboarding/removal runbook</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7487,32 +7522,32 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Reliability requirement.</t>
+          <t>After path validation.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Phase 12</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>On-Premises Kubernetes</t>
+          <t>Final Production Approval</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Document onboarding/removal runbook</t>
+          <t>Final architecture review</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7522,18 +7557,18 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>After path validation.</t>
+          <t>Production gate.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -7547,7 +7582,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Final architecture review</t>
+          <t>Final security review</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7568,7 +7603,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -7582,7 +7617,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Final security review</t>
+          <t>Final IAM review</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7603,7 +7638,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -7617,7 +7652,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Final IAM review</t>
+          <t>Final Model Armor report/decision</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7627,7 +7662,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -7638,7 +7673,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -7652,7 +7687,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Final Model Armor report/decision</t>
+          <t>Final RCA accuracy and confidence evaluation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7662,7 +7697,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -7673,7 +7708,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -7687,7 +7722,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Final RCA accuracy and confidence evaluation</t>
+          <t>Monitoring and alert-delivery validation</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7708,7 +7743,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -7722,7 +7757,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Monitoring and alert-delivery validation</t>
+          <t>Rollback and recovery testing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7743,7 +7778,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -7757,7 +7792,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Rollback and recovery testing</t>
+          <t>Document known limitations and accepted risks</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7767,7 +7802,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -7778,7 +7813,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -7792,7 +7827,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Document known limitations and accepted risks</t>
+          <t>Human approval before production rollout</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -7802,32 +7837,32 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Production gate.</t>
+          <t>Required by design.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Final Production Approval</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Human approval before production rollout</t>
+          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -7841,41 +7876,6 @@
         </is>
       </c>
       <c r="I42" t="inlineStr">
-        <is>
-          <t>Required by design.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>158</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>RCA Output &amp; Evidence</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
         </is>

</xml_diff>

<commit_message>
tracker: row 21 -- PR #183 merged, floor-setting enforcement live, request+response inspection proven (#184)
Records PR #183 (google_model_armor_floorsetting.mcp adopted into Terraform,
enable_floor_setting_enforcement=true applied via CI) and the post-apply E2E
evidence (SanitizeOperationLogEntry shows both request and response inspected
on GOOGLE_MCP_SERVER and AI_PLATFORM, zero regressions). Row stays In Progress
-- SDP, a genuine malicious-payload test, and custom-MCP coverage remain open,
per the same row's existing scope. No duplicate row created.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I60"/>
+  <dimension ref="A1:I61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4493,6 +4493,41 @@
       <c r="I60" t="inlineStr">
         <is>
           <t>CLOSED 2026-08-24. 'Auditable persistence' checked against 4 pillars, each with a file:line or live citation, not assumed: (1) write succeeds -- live-confirmed tonight via gcs.write_evidence spans (ev_001/002/003, ok=true, real bucket/duration_ms). (2) redaction applied before write -- confirmed wired at agent/nodes/evidence_extractor.py:91 (redact(raw) called before write_evidence()), not just a standalone unused function. (3) failure path is auditable -- a permanent GCS write failure writes a structured Cloud Logging event (tests/test_observability.py::test_write_evidence_permanent_failure_writes_structured_log, passing) and now also a gcs.write_evidence span with ok=False (tests/test_gcs_evidence_span.py::test_gcs_span_records_failure_after_retries_exhausted, passing). (4) every write is attributable -- run_id + evidence_id present on both the failure log entry and the live trace span.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>23</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Agent Gateway &amp; Model Armor</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Test Model Armor with Agent Identity, IAP and Agent Gateway</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-24 -- LIVE-VALIDATED. The 2026-08-08 attempt used the GLOBAL Model Armor hostname (modelarmor.googleapis.com) in AuthzExtension.service and got a hard 400 (unsupported Google API for AuthzExtension). This session tried the REGIONAL hostname (modelarmor.us-central1.rep.googleapis.com) instead -- terraform apply succeeded (2 resources created, 0 errors). Ran a real deployed investigation (make smoke) with the wiring live: 33 real gateway requests logged, ALL 33 authorized ALLOWED by the new Model Armor CONTENT_AUTHZ policy (sre-agent-model-armor-gateway-policy), 23 of them actually inspected/processed by Model Armor (processingEffect=CONTENT_MODIFIED, grpcStatus=OK). The 4 non-200 HTTP statuses seen (1x429, 2x404, 1x403) were all pre-existing, unrelated app-level responses (Vertex rate-limit, IAM credential lookups, cluster-config bucket) -- confirmed each still shows model_armor_result=ALLOWED, none were blocked by the new policy. Investigation completed successfully end to end (SMOKE TEST PASSED), no TLS/cert/gateway regression. Branch: test/model-armor-regional-content-authz-trial (committed, NOT merged to main yet -- see row 21/26/131 for what the full trial plan still requires before #30/#32 close: prompt-injection/jailbreak/sensitive-content test cases, full coverage table across all paths, latency measurement, Model Armor Cloud Logging detection-event confirmation).</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4942,7 @@
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Templates exist; live content inspection not active.</t>
+          <t>UPDATED 2026-08-25: PR #183 merged + applied via CI -- google_model_armor_floorsetting.mcp adopted into Terraform (was live drift since 2026-07-13, orphaned from state since commit 9799494 wrongly removed it on a since-disproven gateway-MITM theory -- floor settings are unrelated to the Agent Gateway's own TLS path, verified live). enable_floor_setting_enforcement=true is now PERMANENT and LIVE for both GOOGLE_MCP_SERVER and AI_PLATFORM, both inspect_only=true (inspects + logs, never blocks). Post-apply E2E (2026-08-25 04:08-04:10 UTC) confirms via Model Armor's own SanitizeOperationLogEntry log: BOTH request and response legs inspected on both services (10 GOOGLE_MCP_SERVER entries: 5 request + 5 response; 41 VERTEX_AI entries: 20 request + 21 response), all NO_MATCH_FOUND, zero regressions, zero app errors. Same merge also tore down the Agent Gateway CONTENT_AUTHZ trial (2 resources, explicitly reviewed) -- rejected as the production path since it only ever proved request-side inspection; floor settings proved both directions instead. Still open: a genuine malicious-payload test against floor settings (only benign traffic tested so far), Sensitive Data Protection (not yet added, see docs/management/floor-settings-production-plan-2026-08-25.md), and GOOGLE_MCP_SERVER does NOT cover custom/non-Google MCP servers -- separate, unvalidated path. PR: github.com/AshminPy/sre-agent-gateway/pull/183 (merged, commit 948c510).</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6392,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -6518,7 +6553,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
@@ -6532,7 +6567,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Test Model Armor with Agent Identity, IAP and Agent Gateway</t>
+          <t>Define separate Model Armor policies for input/evidence/output</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -6542,18 +6577,18 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Use supported regional integration.</t>
+          <t>Pending architecture validation.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -6567,7 +6602,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Define separate Model Armor policies for input/evidence/output</t>
+          <t>Test Kubernetes logs/events for false positives</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -6582,13 +6617,13 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Pending architecture validation.</t>
+          <t>Needed before enforcement.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
@@ -6602,7 +6637,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Test Kubernetes logs/events for false positives</t>
+          <t>Confirm Model Armor failure/fallback behaviour</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -6612,32 +6647,32 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Needed before enforcement.</t>
+          <t>Needs explicit failure-mode test.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Phase 2</t>
+          <t>Phase 4</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Agent Gateway &amp; Model Armor</t>
+          <t>Dynamic Investigation &amp; Confidence</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Confirm Model Armor failure/fallback behaviour</t>
+          <t>Confidence calibration testing</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -6647,32 +6682,32 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Needs explicit failure-mode test.</t>
+          <t>Compare confidence with actual RCA accuracy.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>41</v>
+        <v>55</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Phase 4</t>
+          <t>Phase 5</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
+          <t>Testing &amp; Evaluation</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Confidence calibration testing</t>
+          <t>LLM-judge evaluation</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6682,32 +6717,32 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Compare confidence with actual RCA accuracy.</t>
+          <t>Secondary evaluation only.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>55</v>
+        <v>63</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Phase 5</t>
+          <t>Phase 6</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Testing &amp; Evaluation</t>
+          <t>Observability &amp; Reliability</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>LLM-judge evaluation</t>
+          <t>Operational dashboard</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6717,18 +6752,18 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Secondary evaluation only.</t>
+          <t>Needed for operations.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
@@ -6742,7 +6777,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Operational dashboard</t>
+          <t>Controlled delivery test for every alert</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -6752,32 +6787,32 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Needed for operations.</t>
+          <t>Configured alerts must be proven.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Phase 6</t>
+          <t>Phase 7</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Observability &amp; Reliability</t>
+          <t>Multi-Cluster Scalability</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Controlled delivery test for every alert</t>
+          <t>Concurrency/quota/failure-isolation testing</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -6792,27 +6827,27 @@
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Configured alerts must be proven.</t>
+          <t>Scale testing remains.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>76</v>
+        <v>95</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Phase 7</t>
+          <t>Phase 10</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Multi-Cluster Scalability</t>
+          <t>PagerDuty Integration</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Concurrency/quota/failure-isolation testing</t>
+          <t>Design PagerDuty-triggered workflow</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -6822,18 +6857,18 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Scale testing remains.</t>
+          <t>Required Phase 1 integration.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
@@ -6847,7 +6882,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Design PagerDuty-triggered workflow</t>
+          <t>Authenticated Cloud Run webhook receiver</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6862,13 +6897,13 @@
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Required Phase 1 integration.</t>
+          <t>No implementation yet.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
@@ -6882,7 +6917,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Authenticated Cloud Run webhook receiver</t>
+          <t>Pub/Sub buffering and investigation workers</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -6892,18 +6927,18 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>No implementation yet.</t>
+          <t>Planned scalable path.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
@@ -6917,7 +6952,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Pub/Sub buffering and investigation workers</t>
+          <t>Webhook verification and replay protection</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -6927,18 +6962,18 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Planned scalable path.</t>
+          <t>Security requirement.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -6952,7 +6987,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Webhook verification and replay protection</t>
+          <t>Incident deduplication and idempotency</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6967,13 +7002,13 @@
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Security requirement.</t>
+          <t>Production requirement.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -6987,7 +7022,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Incident deduplication and idempotency</t>
+          <t>Trigger read-only investigation from incident</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -7002,13 +7037,13 @@
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Production requirement.</t>
+          <t>Core integration goal.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
@@ -7022,7 +7057,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Trigger read-only investigation from incident</t>
+          <t>Post RCA draft back to PagerDuty</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -7032,32 +7067,32 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Core integration goal.</t>
+          <t>Include evidence/confidence/unknowns/next checks.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Phase 10</t>
+          <t>Phase 11</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>PagerDuty Integration</t>
+          <t>Additional MCP Sources</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Post RCA draft back to PagerDuty</t>
+          <t>Prometheus integration</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -7067,18 +7102,18 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Include evidence/confidence/unknowns/next checks.</t>
+          <t>Future phase.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
@@ -7092,7 +7127,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Prometheus integration</t>
+          <t>Grafana integration</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -7113,7 +7148,7 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
@@ -7127,7 +7162,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Grafana integration</t>
+          <t>Elastic / Elasticsearch integration</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -7148,7 +7183,7 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -7162,7 +7197,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Elastic / Elasticsearch integration</t>
+          <t>Cloud Logging integration</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -7172,18 +7207,18 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Future phase.</t>
+          <t>Future evidence source.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
@@ -7197,7 +7232,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Cloud Logging integration</t>
+          <t>Confluence/runbook integration</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -7207,18 +7242,18 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Future evidence source.</t>
+          <t>Future phase.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -7232,7 +7267,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Confluence/runbook integration</t>
+          <t>GitHub integration</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -7253,7 +7288,7 @@
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -7267,7 +7302,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>GitHub integration</t>
+          <t>Normalized traceable evidence for every source</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -7277,32 +7312,32 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Future phase.</t>
+          <t>Depends on MCP abstraction.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Phase 11</t>
+          <t>Phase 12</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Additional MCP Sources</t>
+          <t>On-Premises Kubernetes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Normalized traceable evidence for every source</t>
+          <t>Custom MCP → Connect Gateway production path</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7312,18 +7347,18 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Depends on MCP abstraction.</t>
+          <t>Production path not proven.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -7337,7 +7372,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Custom MCP → Connect Gateway production path</t>
+          <t>Validate supported agent-authentication model</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7347,18 +7382,18 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Production path not proven.</t>
+          <t>Need short-lived supported auth.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -7372,7 +7407,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Validate supported agent-authentication model</t>
+          <t>Validate IAM and Kubernetes RBAC</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7382,18 +7417,18 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Need short-lived supported auth.</t>
+          <t>Production security requirement.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -7407,7 +7442,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Validate IAM and Kubernetes RBAC</t>
+          <t>Test read-only access to real on-prem cluster</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7417,18 +7452,18 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Production security requirement.</t>
+          <t>Prototype is not production validation.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -7442,7 +7477,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Test read-only access to real on-prem cluster</t>
+          <t>Review audit logs, latency, quotas and isolation</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7457,13 +7492,13 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Prototype is not production validation.</t>
+          <t>Reliability requirement.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -7477,7 +7512,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Review audit logs, latency, quotas and isolation</t>
+          <t>Document onboarding/removal runbook</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7487,32 +7522,32 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Reliability requirement.</t>
+          <t>After path validation.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Phase 12</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>On-Premises Kubernetes</t>
+          <t>Final Production Approval</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Document onboarding/removal runbook</t>
+          <t>Final architecture review</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7522,18 +7557,18 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>After path validation.</t>
+          <t>Production gate.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -7547,7 +7582,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Final architecture review</t>
+          <t>Final security review</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7568,7 +7603,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -7582,7 +7617,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Final security review</t>
+          <t>Final IAM review</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7603,7 +7638,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -7617,7 +7652,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Final IAM review</t>
+          <t>Final Model Armor report/decision</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7627,7 +7662,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -7638,7 +7673,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -7652,7 +7687,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Final Model Armor report/decision</t>
+          <t>Final RCA accuracy and confidence evaluation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7662,7 +7697,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -7673,7 +7708,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -7687,7 +7722,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Final RCA accuracy and confidence evaluation</t>
+          <t>Monitoring and alert-delivery validation</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7708,7 +7743,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -7722,7 +7757,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Monitoring and alert-delivery validation</t>
+          <t>Rollback and recovery testing</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7743,7 +7778,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -7757,7 +7792,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Rollback and recovery testing</t>
+          <t>Document known limitations and accepted risks</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7767,7 +7802,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -7778,7 +7813,7 @@
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
@@ -7792,7 +7827,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Document known limitations and accepted risks</t>
+          <t>Human approval before production rollout</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -7802,32 +7837,32 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Production gate.</t>
+          <t>Required by design.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Final Production Approval</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Human approval before production rollout</t>
+          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -7841,41 +7876,6 @@
         </is>
       </c>
       <c r="I42" t="inlineStr">
-        <is>
-          <t>Required by design.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>158</v>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>RCA Output &amp; Evidence</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I43" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
         </is>

</xml_diff>

<commit_message>
tracker: close #85 (live-tested), file #203 + #206, correct #32/#164/#79 notes
Real drift found during today's issue audit: 5 changes queued this session
never actually landed in the tracker earlier -- caught and applied now, plus
today's new #206 fix.

- Row 122 (#32/Model Armor): corrected -- app-level path is structurally
  dead code, cause filed separately as #203, blocked on #30.
- Row 123 (#79/supply chain): dorny/paths-filter is now SHA-pinned, 2 of 3
  gaps remain.
- New Completed row 164: #85 closed as not-planned, contradicted by a real
  2026-08-25 live test.
- New Not Started row 165: #203 filed (Model Armor gating root cause).
- New In Progress row 166: #206 (resource_identity_match false positive),
  fix merged via PR #207, live re-validation still pending.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I61"/>
+  <dimension ref="A1:I62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4528,6 +4528,41 @@
       <c r="I61" t="inlineStr">
         <is>
           <t>CLOSED 2026-08-24 -- LIVE-VALIDATED. The 2026-08-08 attempt used the GLOBAL Model Armor hostname (modelarmor.googleapis.com) in AuthzExtension.service and got a hard 400 (unsupported Google API for AuthzExtension). This session tried the REGIONAL hostname (modelarmor.us-central1.rep.googleapis.com) instead -- terraform apply succeeded (2 resources created, 0 errors). Ran a real deployed investigation (make smoke) with the wiring live: 33 real gateway requests logged, ALL 33 authorized ALLOWED by the new Model Armor CONTENT_AUTHZ policy (sre-agent-model-armor-gateway-policy), 23 of them actually inspected/processed by Model Armor (processingEffect=CONTENT_MODIFIED, grpcStatus=OK). The 4 non-200 HTTP statuses seen (1x429, 2x404, 1x403) were all pre-existing, unrelated app-level responses (Vertex rate-limit, IAM credential lookups, cluster-config bucket) -- confirmed each still shows model_armor_result=ALLOWED, none were blocked by the new policy. Investigation completed successfully end to end (SMOKE TEST PASSED), no TLS/cert/gateway regression. Branch: test/model-armor-regional-content-authz-trial (committed, NOT merged to main yet -- see row 21/26/131 for what the full trial plan still requires before #30/#32 close: prompt-injection/jailbreak/sensitive-content test cases, full coverage table across all paths, latency measurement, Model Armor Cloud Logging detection-event confirmation).</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>164</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Phase 1</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Production Readiness</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>Issue #85: Custom Cloud Run MCP fallback confirmed operational (issue closed as not-planned)</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>P2-medium-fix</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>CLOSED 2026-08-27 as not-planned -- the issue's premise was contradicted by a real live test. #85 was filed 2026-08-10 from a static code/Terraform read claiming the custom Cloud Run MCP fallback could not build a k8s client and had no reachable connectivity path. On 2026-08-25 the path was exercised for real (PRs #193/#194: gke_remote_mcp's URL temporarily broken to force fallback, deployed via normal CI, then reverted the same way). CI's own smoke test -- not a staged local run -- returned primary_mcp_source='gke_remote_mcp', actual_mcp_sources=['k8s_mcp'], passed. Evidence: docs/management/custom-mcp-model-armor-coverage-2026-08-25.md. DOES NOT cover: the fallback is unprotected -- that traffic transits the Agent Gateway but Model Armor does not inspect it (0 GOOGLE_MCP_SERVER vs 12 VERTEX_AI log entries in the same window); tracked separately. Multi-cluster half of #85's body (single global K8S_MCP_URL, mcp/server.py:78 @lru_cache(maxsize=1), no per-cluster mcp_url in variables.tf) moved to #86 -- verified still present on main today, NOT fixed by this closure.</t>
         </is>
       </c>
     </row>
@@ -4542,7 +4577,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I52"/>
+  <dimension ref="A1:I53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -6272,7 +6307,7 @@
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>Not active in live path.</t>
+          <t>UPDATED 2026-08-27: root cause of 'not active in live path' now identified and filed as GitHub #203. agent/main.py:909 returns early unless MODEL_ARMOR_TEMPLATE is set, and iac/agent/agent_engine.tf:102-108 sets that env var ONLY when var.enable_agent_gateway is false; variables.tf:103-106 defaults it to true with no CI override. So app-level Model Armor (_sanitize) is unreachable in every real deploy -- input sanitization at main.py:1150 and the #32 output-verdict path at main.py:1253-1264 (content_flagged / requires_human_review) have never executed in production. The gating comment justifies this as redundant with a gateway CONTENT_AUTHZ Model Armor extension, but agent_gateway.tf:5-8 states no working Terraform path to wire that ever existed (real API rejection), and the only google_network_services_authz_extension on main is 'iap'. Blocked by #30 (endpoint hostname registration must be fixed before re-enabling). Verified against main @ 2384d21.</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6342,7 @@
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>Pinning/CI/container hardening remain.</t>
+          <t>UPDATED 2026-08-27 (verified against main @ 2384d21, GitHub #79). PARTIALLY DONE: dorny/paths-filter is now pinned to a full commit SHA (.github/workflows/terraform-apply.yml:48, ceb8a2b8f2d89434be7ff52d3de7ec3738c5cc9d # v4.0.3). REMAINING, all confirmed still present: (1) every other action is pinned by tag not SHA -- actions/checkout@v4 (and @v6 in claude-review-response.yml:101), actions/setup-python@v5, google-github-actions/auth@v2, hashicorp/setup-terraform@v3, anthropics/claude-code-action@v1, across all 5 workflows; (2) no Python lock file anywhere -- agent/requirements.txt and mcp/requirements.txt still use &gt;= ranges; (3) mcp/Dockerfile has no USER directive (runs as root) and line 6 is still an unpinned 'RUN pip install uv'. Item 3 is the cheapest and highest-value of the three: a USER line plus a pinned uv version, no CI or dependency-resolution risk.</t>
         </is>
       </c>
     </row>
@@ -6378,6 +6413,41 @@
       <c r="I52" t="inlineStr">
         <is>
           <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). STILL NOT live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which has not occurred naturally yet (waiting, per 2026-08-23 decision). Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. RESOLVED 2026-08-24: the resource.type sub-item is done -- live-confirmed via `gcloud monitoring policies list --project=sreagent-t2-demo`, all 5 alerts (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) now filter on resource.type="cloud_run_revision" (PR #178, merged + deployed, CI run 32694669742). See row 163 for the alert fix's own tracking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>166</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Issue #206: resource_identity_match scored 0.0 on an unambiguous case -- trusted LLM free text instead of real evidence</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>In Progress</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>MERGED 2026-08-27, PR #207. Real live run (run_20260827_182635_yfcm, imagepull scenario) scored root_cause_confidence 0.74/review_required despite a textbook-unambiguous case -- resource_identity_match (20% weight) hit 0.0. Verified via the real GCS evidence bucket: all 3 raw evidence items explicitly named test-incidents/imagepull-pod, so the mismatch was not real. Root cause: evidence_extractor.py wrote resource_id from the extractor LLM's own free-text description (never validated), and scorer.py's resource_identity_match does a plain substring check against it -- a wording mismatch, not an evidence mismatch, could trigger the penalty. Same bug CLASS as PR #204's 16 fixes (real data must not be conflated with model-generated text feeding a score), a 17th instance PR #204 didn't cover. Fix: resource_id is now built deterministically from the real tool-call arguments (state['tool_history'][-1]['args']), per the verified schema (toolspec.json for gke_remote_mcp, mcp/server.py's @guarded(...) decorators for custom MCP) -- never LLM-written text. 3 new regression tests, full suite 349/349, ruff clean. STILL OPEN: live re-validation -- rerun the same imagepull scenario post-deploy and confirm resource_identity_match scores 1.0 on this exact case. Move to Completed only after that live check passes.</t>
         </is>
       </c>
     </row>
@@ -6392,7 +6462,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -7878,6 +7948,41 @@
       <c r="I42" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>165</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Phase 2</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Agent Gateway &amp; Model Armor</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Issue #203: MODEL_ARMOR_TEMPLATE gated on gateway-OFF, so app-level Model Armor is dead code in every real deploy</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>FILED 2026-08-27. Cause behind row 122's 'not active in live path' and the reason #32 cannot be validated as written. Fix: set MODEL_ARMOR_TEMPLATE unconditionally instead of gating on var.enable_agent_gateway, and correct the two stale comments (agent_engine.tf:103, model_armor.tf:12) that justify the gate by citing a gateway-side CONTENT_AUTHZ Model Armor extension that does not exist. BLOCKED BY #30 -- the endpoint hostname registration must be fixed before re-enabling (agent/main.py:876 uses modelarmor.{REGION}.rep.googleapis.com; #30 reports Agent Registry has the non-.rep. host; needs a live gcloud alpha agent-registry services list check to confirm, not verifiable from the repo). OPEN DESIGN QUESTION, decide before enabling: what happens when _sanitize() flags something -- current code blocks/replaces the text, and pi_and_jailbreak at MEDIUM_AND_ABOVE has false-positived 3 times on ordinary SRE text in one evening (see #202). A false positive here corrupts a legitimate RCA summary.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: #206 live-validated, moved In Progress -> Completed
Re-ran the exact scenario that exposed the bug: resource_identity_match
0.0 -> 1.0 on a real deployed run, not just unit tests. Overall confidence
0.74 -> 0.835. Still in review band, but now for unrelated real reasons.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4563,6 +4563,41 @@
       <c r="I62" t="inlineStr">
         <is>
           <t>CLOSED 2026-08-27 as not-planned -- the issue's premise was contradicted by a real live test. #85 was filed 2026-08-10 from a static code/Terraform read claiming the custom Cloud Run MCP fallback could not build a k8s client and had no reachable connectivity path. On 2026-08-25 the path was exercised for real (PRs #193/#194: gke_remote_mcp's URL temporarily broken to force fallback, deployed via normal CI, then reverted the same way). CI's own smoke test -- not a staged local run -- returned primary_mcp_source='gke_remote_mcp', actual_mcp_sources=['k8s_mcp'], passed. Evidence: docs/management/custom-mcp-model-armor-coverage-2026-08-25.md. DOES NOT cover: the fallback is unprotected -- that traffic transits the Agent Gateway but Model Armor does not inspect it (0 GOOGLE_MCP_SERVER vs 12 VERTEX_AI log entries in the same window); tracked separately. Multi-cluster half of #85's body (single global K8S_MCP_URL, mcp/server.py:78 @lru_cache(maxsize=1), no per-cluster mcp_url in variables.tf) moved to #86 -- verified still present on main today, NOT fixed by this closure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>166</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Issue #206: resource_identity_match scored 0.0 on an unambiguous case -- trusted LLM free text instead of real evidence</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LIVE-VALIDATED 2026-08-27. Deployed via terraform-apply run 33108575687 (apply 6m34s, smoke test passed). Re-ran the exact same imagepull scenario (run_20260827_205724_odwb) that originally exposed the bug: root_cause_confidence.components.resource_identity_match went from 0.0 to 1.0 -- the predicted fix, confirmed against a real deployed run, not just unit tests. Overall confidence moved 0.74 -&gt; 0.835. Investigation stayed in the REVIEW band, but now for unrelated, legitimate reasons (direct_support 0.5 -- 2 of 4 claims are inference rather than independently grounded fact; one claim on '0 restarts' scored weak_overlap) -- not a regression, a different, real scoring signal working as designed.</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -6413,41 +6448,6 @@
       <c r="I52" t="inlineStr">
         <is>
           <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). STILL NOT live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which has not occurred naturally yet (waiting, per 2026-08-23 decision). Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. RESOLVED 2026-08-24: the resource.type sub-item is done -- live-confirmed via `gcloud monitoring policies list --project=sreagent-t2-demo`, all 5 alerts (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) now filter on resource.type="cloud_run_revision" (PR #178, merged + deployed, CI run 32694669742). See row 163 for the alert fix's own tracking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>166</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Issue #206: resource_identity_match scored 0.0 on an unambiguous case -- trusted LLM free text instead of real evidence</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>MERGED 2026-08-27, PR #207. Real live run (run_20260827_182635_yfcm, imagepull scenario) scored root_cause_confidence 0.74/review_required despite a textbook-unambiguous case -- resource_identity_match (20% weight) hit 0.0. Verified via the real GCS evidence bucket: all 3 raw evidence items explicitly named test-incidents/imagepull-pod, so the mismatch was not real. Root cause: evidence_extractor.py wrote resource_id from the extractor LLM's own free-text description (never validated), and scorer.py's resource_identity_match does a plain substring check against it -- a wording mismatch, not an evidence mismatch, could trigger the penalty. Same bug CLASS as PR #204's 16 fixes (real data must not be conflated with model-generated text feeding a score), a 17th instance PR #204 didn't cover. Fix: resource_id is now built deterministically from the real tool-call arguments (state['tool_history'][-1]['args']), per the verified schema (toolspec.json for gke_remote_mcp, mcp/server.py's @guarded(...) decorators for custom MCP) -- never LLM-written text. 3 new regression tests, full suite 349/349, ruff clean. STILL OPEN: live re-validation -- rerun the same imagepull scenario post-deploy and confirm resource_identity_match scores 1.0 on this exact case. Move to Completed only after that live check passes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: #206 live-validated, moved In Progress -> Completed (#208)
Re-ran the exact scenario that exposed the bug: resource_identity_match
0.0 -> 1.0 on a real deployed run, not just unit tests. Overall confidence
0.74 -> 0.835. Still in review band, but now for unrelated real reasons.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I62"/>
+  <dimension ref="A1:I63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4563,6 +4563,41 @@
       <c r="I62" t="inlineStr">
         <is>
           <t>CLOSED 2026-08-27 as not-planned -- the issue's premise was contradicted by a real live test. #85 was filed 2026-08-10 from a static code/Terraform read claiming the custom Cloud Run MCP fallback could not build a k8s client and had no reachable connectivity path. On 2026-08-25 the path was exercised for real (PRs #193/#194: gke_remote_mcp's URL temporarily broken to force fallback, deployed via normal CI, then reverted the same way). CI's own smoke test -- not a staged local run -- returned primary_mcp_source='gke_remote_mcp', actual_mcp_sources=['k8s_mcp'], passed. Evidence: docs/management/custom-mcp-model-armor-coverage-2026-08-25.md. DOES NOT cover: the fallback is unprotected -- that traffic transits the Agent Gateway but Model Armor does not inspect it (0 GOOGLE_MCP_SERVER vs 12 VERTEX_AI log entries in the same window); tracked separately. Multi-cluster half of #85's body (single global K8S_MCP_URL, mcp/server.py:78 @lru_cache(maxsize=1), no per-cluster mcp_url in variables.tf) moved to #86 -- verified still present on main today, NOT fixed by this closure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>166</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>Issue #206: resource_identity_match scored 0.0 on an unambiguous case -- trusted LLM free text instead of real evidence</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LIVE-VALIDATED 2026-08-27. Deployed via terraform-apply run 33108575687 (apply 6m34s, smoke test passed). Re-ran the exact same imagepull scenario (run_20260827_205724_odwb) that originally exposed the bug: root_cause_confidence.components.resource_identity_match went from 0.0 to 1.0 -- the predicted fix, confirmed against a real deployed run, not just unit tests. Overall confidence moved 0.74 -&gt; 0.835. Investigation stayed in the REVIEW band, but now for unrelated, legitimate reasons (direct_support 0.5 -- 2 of 4 claims are inference rather than independently grounded fact; one claim on '0 restarts' scored weak_overlap) -- not a regression, a different, real scoring signal working as designed.</t>
         </is>
       </c>
     </row>
@@ -4577,7 +4612,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I53"/>
+  <dimension ref="A1:I52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -6413,41 +6448,6 @@
       <c r="I52" t="inlineStr">
         <is>
           <t>Same _use_grpc=False fix as row 152's rca_builder.py resolution, applied to the 3 sibling call sites sharing the identical pattern (sre-agent-tool-failures, sre-agent-routing-failures, sre-agent-evidence-storage-failures). PR #175 merged and deployed (CI run 32653113035, smoke test passed). STILL NOT live-validated -- these 3 only write on a genuine tool/routing/evidence-storage failure, which has not occurred naturally yet (waiting, per 2026-08-23 decision). Completion requires: a real failure of each kind occurring live with the corresponding log entry confirmed written, no 403. RESOLVED 2026-08-24: the resource.type sub-item is done -- live-confirmed via `gcloud monitoring policies list --project=sreagent-t2-demo`, all 5 alerts (gke_mcp_failures, custom_mcp_failures, repeated_tool_failures, routing_failures, evidence_storage_failures) now filter on resource.type="cloud_run_revision" (PR #178, merged + deployed, CI run 32694669742). See row 163 for the alert fix's own tracking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="n">
-        <v>166</v>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>Phase 4</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>Dynamic Investigation &amp; Confidence</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>Issue #206: resource_identity_match scored 0.0 on an unambiguous case -- trusted LLM free text instead of real evidence</t>
-        </is>
-      </c>
-      <c r="E53" t="inlineStr">
-        <is>
-          <t>In Progress</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="I53" t="inlineStr">
-        <is>
-          <t>MERGED 2026-08-27, PR #207. Real live run (run_20260827_182635_yfcm, imagepull scenario) scored root_cause_confidence 0.74/review_required despite a textbook-unambiguous case -- resource_identity_match (20% weight) hit 0.0. Verified via the real GCS evidence bucket: all 3 raw evidence items explicitly named test-incidents/imagepull-pod, so the mismatch was not real. Root cause: evidence_extractor.py wrote resource_id from the extractor LLM's own free-text description (never validated), and scorer.py's resource_identity_match does a plain substring check against it -- a wording mismatch, not an evidence mismatch, could trigger the penalty. Same bug CLASS as PR #204's 16 fixes (real data must not be conflated with model-generated text feeding a score), a 17th instance PR #204 didn't cover. Fix: resource_id is now built deterministically from the real tool-call arguments (state['tool_history'][-1]['args']), per the verified schema (toolspec.json for gke_remote_mcp, mcp/server.py's @guarded(...) decorators for custom MCP) -- never LLM-written text. 3 new regression tests, full suite 349/349, ruff clean. STILL OPEN: live re-validation -- rerun the same imagepull scenario post-deploy and confirm resource_identity_match scores 1.0 on this exact case. Move to Completed only after that live check passes.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: close #209 (wrong-target routing) and #211 (sidecar logs)
Both merged and deployed today. #209 live-validated against the exact
failing case. #211 tested against a synthetic 2-container pod, not
real Istio -- caveat recorded, not overclaimed as fully proven.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4598,6 +4598,76 @@
       <c r="I63" t="inlineStr">
         <is>
           <t>LIVE-VALIDATED 2026-08-27. Deployed via terraform-apply run 33108575687 (apply 6m34s, smoke test passed). Re-ran the exact same imagepull scenario (run_20260827_205724_odwb) that originally exposed the bug: root_cause_confidence.components.resource_identity_match went from 0.0 to 1.0 -- the predicted fix, confirmed against a real deployed run, not just unit tests. Overall confidence moved 0.74 -&gt; 0.835. Investigation stayed in the REVIEW band, but now for unrelated, legitimate reasons (direct_support 0.5 -- 2 of 4 claims are inference rather than independently grounded fact; one claim on '0 restarts' scored weak_overlap) -- not a regression, a different, real scoring signal working as designed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>167</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Issue #209: task_planner/mcp_router never saw the original query -- blank Pod hint caused the agent to investigate the wrong resource entirely</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>MERGED and DEPLOYED 2026-08-27 (PR #210, terraform-apply run succeeded, smoke test passed). Found during confidence-calibration baseline work: a real test case ('notification-svc shows no endpoints', no pod hint) investigated a completely unrelated pod's missing ConfigMap instead, scoring it 0.95 confidence -- high confidence, wrong incident. Root cause: task_planner/mcp_router only ever saw normalized namespace/pod fields, never the original incident report; a blank pod left no way to recover the real target, so the first tool call went unscoped across the whole (busy) namespace and locked onto whatever was loudest. Fix: thread user_query into both prompts, with explicit scoping instructions. LIVE-VALIDATED: re-ran the exact same case after the fix -- correctly targeted notification-svc. 2 new regression tests, full suite 352/352 at merge time. Surfaced a second, narrower issue (wrong resourceType guess + over-weighted a resulting NotFound into a false conclusion) -- not fixed here, needs its own pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>168</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Issue #211: get_k8s_logs silently dropped the container argument -- Istio/sidecar pods default to the wrong container's logs</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>MERGED and DEPLOYED 2026-08-27 (PR #212, terraform-apply run succeeded, smoke test passed). User-reported: real work-environment pods run with an Istio sidecar, and the agent was seen investigating the wrong container. Reproduced live against a real 2-container test pod (istio-proxy + app): with no container argument forwarded, Kubernetes itself defaulted to the sidecar -- confirmed via the real API response 'Defaulted container "istio-proxy" out of: istio-proxy, app'. Root cause: agent/mcp_client.py's request builder silently dropped `container` even when supplied, and no tool description ever told the model it was an option. Fix: forward container through, expose it in both MCP tool descriptions, add explicit SIDECAR guidance (check container list first, prefer the app container over common sidecar/infra names) to the router prompt. 3 new regression tests (deterministic, on the request builder itself), full suite 355/355. CAVEAT, not yet closed further: tested against a synthetic 2-container pod, not a real Istio-injected one -- no Istio installed in this test cluster. The code fix and the live Kubernetes default-container behavior are both confirmed real; a genuine istio-proxy sidecar has not been used to verify end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
tracker: close #209 (wrong-target routing) and #211 (sidecar logs) (#213)
Both merged and deployed today. #209 live-validated against the exact
failing case. #211 tested against a synthetic 2-container pod, not
real Istio -- caveat recorded, not overclaimed as fully proven.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I63"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4598,6 +4598,76 @@
       <c r="I63" t="inlineStr">
         <is>
           <t>LIVE-VALIDATED 2026-08-27. Deployed via terraform-apply run 33108575687 (apply 6m34s, smoke test passed). Re-ran the exact same imagepull scenario (run_20260827_205724_odwb) that originally exposed the bug: root_cause_confidence.components.resource_identity_match went from 0.0 to 1.0 -- the predicted fix, confirmed against a real deployed run, not just unit tests. Overall confidence moved 0.74 -&gt; 0.835. Investigation stayed in the REVIEW band, but now for unrelated, legitimate reasons (direct_support 0.5 -- 2 of 4 claims are inference rather than independently grounded fact; one claim on '0 restarts' scored weak_overlap) -- not a regression, a different, real scoring signal working as designed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>167</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>Issue #209: task_planner/mcp_router never saw the original query -- blank Pod hint caused the agent to investigate the wrong resource entirely</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>MERGED and DEPLOYED 2026-08-27 (PR #210, terraform-apply run succeeded, smoke test passed). Found during confidence-calibration baseline work: a real test case ('notification-svc shows no endpoints', no pod hint) investigated a completely unrelated pod's missing ConfigMap instead, scoring it 0.95 confidence -- high confidence, wrong incident. Root cause: task_planner/mcp_router only ever saw normalized namespace/pod fields, never the original incident report; a blank pod left no way to recover the real target, so the first tool call went unscoped across the whole (busy) namespace and locked onto whatever was loudest. Fix: thread user_query into both prompts, with explicit scoping instructions. LIVE-VALIDATED: re-ran the exact same case after the fix -- correctly targeted notification-svc. 2 new regression tests, full suite 352/352 at merge time. Surfaced a second, narrower issue (wrong resourceType guess + over-weighted a resulting NotFound into a false conclusion) -- not fixed here, needs its own pass.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>168</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Phase 4</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Dynamic Investigation &amp; Confidence</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Issue #211: get_k8s_logs silently dropped the container argument -- Istio/sidecar pods default to the wrong container's logs</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>MERGED and DEPLOYED 2026-08-27 (PR #212, terraform-apply run succeeded, smoke test passed). User-reported: real work-environment pods run with an Istio sidecar, and the agent was seen investigating the wrong container. Reproduced live against a real 2-container test pod (istio-proxy + app): with no container argument forwarded, Kubernetes itself defaulted to the sidecar -- confirmed via the real API response 'Defaulted container "istio-proxy" out of: istio-proxy, app'. Root cause: agent/mcp_client.py's request builder silently dropped `container` even when supplied, and no tool description ever told the model it was an option. Fix: forward container through, expose it in both MCP tool descriptions, add explicit SIDECAR guidance (check container list first, prefer the app container over common sidecar/infra names) to the router prompt. 3 new regression tests (deterministic, on the request builder itself), full suite 355/355. CAVEAT, not yet closed further: tested against a synthetic 2-container pod, not a real Istio-injected one -- no Istio installed in this test cluster. The code fix and the live Kubernetes default-container behavior are both confirmed real; a genuine istio-proxy sidecar has not been used to verify end-to-end.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): mark Connect Gateway production path Completed
Row 110 moved from Not Started to Completed with full evidence:
production path proven end-to-end, including the real CI regression
found and fixed (PR #243) and a real post-CI live investigation.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -2377,7 +2377,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I64"/>
+  <dimension ref="A1:I65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -4633,6 +4633,41 @@
       <c r="I64" t="inlineStr">
         <is>
           <t>MERGED and DEPLOYED 2026-08-27 (PR #212, terraform-apply run succeeded, smoke test passed). User-reported: real work-environment pods run with an Istio sidecar, and the agent was seen investigating the wrong container. Reproduced live against a real 2-container test pod (istio-proxy + app): with no container argument forwarded, Kubernetes itself defaulted to the sidecar -- confirmed via the real API response 'Defaulted container "istio-proxy" out of: istio-proxy, app'. Root cause: agent/mcp_client.py's request builder silently dropped `container` even when supplied, and no tool description ever told the model it was an option. Fix: forward container through, expose it in both MCP tool descriptions, add explicit SIDECAR guidance (check container list first, prefer the app container over common sidecar/infra names) to the router prompt. 3 new regression tests (deterministic, on the request builder itself), full suite 355/355. CAVEAT, not yet closed further: tested against a synthetic 2-container pod, not a real Istio-injected one -- no Istio installed in this test cluster. The code fix and the live Kubernetes default-container behavior are both confirmed real; a genuine istio-proxy sidecar has not been used to verify end-to-end.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>110</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Phase 12</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>On-Premises Kubernetes</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>Custom MCP → Connect Gateway production path</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>COMPLETED 2026-09-05. Production path proven end-to-end, including a real regression found and fixed along the way: PR #242's merge caused CI's first terraform-apply on main to silently destroy the Connect Gateway IAM binding (roles/gkehub.gatewayReader) and the Cloud Run K8S_MCP_KUBE_CONTEXT env var, because CI never passed onprem_fleet_membership/custom_mcp_kube_context and the underlying Terraform resource required a kubeconfig CI never legitimately has. Fixed structurally in PR #243, not just patched: Kubernetes RBAC moved to a separate repo (AshminPy/sre-k8s-rbac, mirroring the work-side ownership model -- reusable ClusterRoles + per-cluster bindings, CI does static validation only, never holds a cluster credential); Fleet/Connect Agent bootstrap is now an explicit manual operator step; sre-agent-gateway's Terraform no longer needs kubeconfig access at all. A real, pre-existing RBAC gap was found and fixed along the way: the built-in `view` ClusterRole does not grant `nodes` (get/list), which list_nodes/describe_node require -- confirmed against this repo's own PRODUCTION-LAUNCH-PLAN.md history and fixed in the new sre-agent-reader ClusterRole. Live-proven: a real CI apply on main (post-fix) left the IAM binding and env var intact, and a real post-CI investigation (run_20260905_154124_fdvw) completed successfully through the full path Agent -&gt; Agent Gateway -&gt; Custom MCP -&gt; Connect Gateway -&gt; sre-lab, with 3 real tool calls, complete evidence coverage, and a correct grounded conclusion. Final terraform plan: 0 to add, 0 to destroy. See PHASE1_EVIDENCE_LOG.md for full detail.</t>
         </is>
       </c>
     </row>
@@ -6567,7 +6602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="4" max="4"/>
@@ -7498,7 +7533,7 @@
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -7512,7 +7547,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Custom MCP → Connect Gateway production path</t>
+          <t>Validate supported agent-authentication model</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -7522,18 +7557,18 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Production path not proven.</t>
+          <t>Need short-lived supported auth.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
@@ -7547,7 +7582,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Validate supported agent-authentication model</t>
+          <t>Validate IAM and Kubernetes RBAC</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -7557,18 +7592,18 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Need short-lived supported auth.</t>
+          <t>Production security requirement.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
@@ -7582,7 +7617,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Validate IAM and Kubernetes RBAC</t>
+          <t>Test read-only access to real on-prem cluster</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -7592,18 +7627,18 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Production security requirement.</t>
+          <t>Prototype is not production validation.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -7617,7 +7652,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Test read-only access to real on-prem cluster</t>
+          <t>Review audit logs, latency, quotas and isolation</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -7632,13 +7667,13 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Prototype is not production validation.</t>
+          <t>Reliability requirement.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
@@ -7652,7 +7687,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Review audit logs, latency, quotas and isolation</t>
+          <t>Document onboarding/removal runbook</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -7662,32 +7697,32 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Reliability requirement.</t>
+          <t>After path validation.</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>115</v>
+        <v>128</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Phase 12</t>
+          <t>Final</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>On-Premises Kubernetes</t>
+          <t>Final Production Approval</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Document onboarding/removal runbook</t>
+          <t>Final architecture review</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -7697,18 +7732,18 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>After path validation.</t>
+          <t>Production gate.</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
@@ -7722,7 +7757,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Final architecture review</t>
+          <t>Final security review</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -7743,7 +7778,7 @@
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -7757,7 +7792,7 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Final security review</t>
+          <t>Final IAM review</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -7778,7 +7813,7 @@
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
@@ -7792,7 +7827,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Final IAM review</t>
+          <t>Final Model Armor report/decision</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -7802,7 +7837,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -7813,7 +7848,7 @@
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
@@ -7827,7 +7862,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Final Model Armor report/decision</t>
+          <t>Final RCA accuracy and confidence evaluation</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -7837,7 +7872,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
@@ -7848,7 +7883,7 @@
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
@@ -7862,7 +7897,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Final RCA accuracy and confidence evaluation</t>
+          <t>Monitoring and alert-delivery validation</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -7883,7 +7918,7 @@
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
@@ -7897,7 +7932,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Monitoring and alert-delivery validation</t>
+          <t>Rollback and recovery testing</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -7918,7 +7953,7 @@
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
@@ -7932,7 +7967,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Rollback and recovery testing</t>
+          <t>Document known limitations and accepted risks</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -7942,7 +7977,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -7953,7 +7988,7 @@
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
@@ -7967,7 +8002,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Document known limitations and accepted risks</t>
+          <t>Human approval before production rollout</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -7977,32 +8012,32 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Production gate.</t>
+          <t>Required by design.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>136</v>
+        <v>158</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Final</t>
+          <t>Phase 3</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Final Production Approval</t>
+          <t>RCA Output &amp; Evidence</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Human approval before production rollout</t>
+          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -8016,41 +8051,6 @@
         </is>
       </c>
       <c r="I41" t="inlineStr">
-        <is>
-          <t>Required by design.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>158</v>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>Phase 3</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>RCA Output &amp; Evidence</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Container-aware evidence collection and attribution (multi-container/sidecar pods)</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>Not Started</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>Critical</t>
-        </is>
-      </c>
-      <c r="I42" t="inlineStr">
         <is>
           <t>Confirmed 2026-08-21/22: ALL workloads on the target GKE Autopilot clusters run an Istio sidecar -- this affects every investigation, not an edge case. Confirmed gap, 3 layers, read directly from code: (1) agent/mcp_client.py:306-317's GKE Remote MCP payload builder for get_k8s_logs never forwards a container argument even though the API supports one (custom MCP's mcp/tools/logs.py already does this correctly); (2) agent/nodes/evidence_extractor.py's evidence schema has no container field and never surfaces describe_pod_detail's own containers/container_statuses into the evidence the LLM reasons over; (3) agent/prompts.py's tool-selection prompt has no language teaching the model that a pod can have multiple containers, and mcp_router.py's auto-fill only ever sets namespace/pod. Scope, deliberately narrow -- data plumbing and prompt fix, not a redesign: forward the container arg on the GKE path, surface containers/container_statuses into key_facts, add container-selection guidance to the tool-selection prompt, add a container field to the evidence schema. Required before Milestone 1 (GKE pilot) per management direction 2026-08-22 -- every pilot target has this. See EXT-003 (External Dependencies worksheet) for the corresponding real work-cluster observation.</t>
         </is>

</xml_diff>

<commit_message>
docs(tracker): record PR #249 evidence on rows 121/165 (#203)
Evidence-only update, no status change on either row -- neither row's
scope maps 1:1 to PR #249 alone:

- Row 165 (ties GitHub #203): PR #249 shipped a compensating control
  (mcp/response_guard.py) for the RESPONSE_BODY gap on the custom MCP
  path specifically, but GKE Remote MCP's identical gap remains
  uncompensated and the Google support case this row already committed
  to filing is still not filed -- issue stays open, row stays
  'Waiting on Google Support'.
- Row 121 ('Agent Gateway security validation'): PR #249 made the
  REQUEST_AUTHZ fail-closed fix durable (authz_fail_open default
  true -> false, merged + deployed, confirmed live). Row covers more
  than this one fix (CONTENT_AUTHZ response-side gap, row 165, remains
  open) -- stays 'In Progress'.

Full evidence also posted as a GitHub comment on issue #203.
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -6377,7 +6377,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Final production review. | UPDATE 2026-09-05: REQUEST_AUTHZ staleness/bypass test completed -- revoked the agent identity's roles/iap.egressor binding on an already-warm (&gt;5h) connection, retried immediately: denied within 2.8s, gateway log shows authzPolicyInfo.result=DENIED on the very first egress attempt, zero stale-enforcement window. Restored, confirmed access works again, confirmed zero Terraform drift. Verdict: PASS, no bypass, confirmed against official Google docs (authz extensions invoke live at the request-headers stage, no cache). See PHASE1_EVIDENCE_LOG.md.</t>
+          <t>Final production review. | UPDATE 2026-09-05: REQUEST_AUTHZ staleness/bypass test completed -- revoked the agent identity's roles/iap.egressor binding on an already-warm (&gt;5h) connection, retried immediately: denied within 2.8s, gateway log shows authzPolicyInfo.result=DENIED on the very first egress attempt, zero stale-enforcement window. Restored, confirmed access works again, confirmed zero Terraform drift. Verdict: PASS, no bypass, confirmed against official Google docs (authz extensions invoke live at the request-headers stage, no cache). See PHASE1_EVIDENCE_LOG.md. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z): the REQUEST_AUTHZ staleness/bypass test above (2026-09-05) was investigation-only -- authz_fail_open was still true by default. This PR makes the fix durable: iac/agent/variables.tf's authz_fail_open default changed true -&gt; false, merged, deployed via CI (run 34054067651), confirmed live via `terraform state show` (google_network_services_authz_extension.iap[0].fail_open = false). Not independently re-tested post-merge beyond confirming the live value (the underlying revoke/retry/no-bypass behavior was already proven 2026-09-05 against the same mechanism). NOT marking this row Completed -- 'Agent Gateway security validation' / 'Final Agent Gateway production validation' covers more than this one fix (CONTENT_AUTHZ response-side gap, row 165/#203, remains open).</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>UPDATED 2026-09-05. Investigated end to end on feat/phase-1-release. Fixed the original gating bug this row describes, plus corrected agent_gateway.tf's stale comment (the gateway-side CONTENT_AUTHZ extension DOES exist on the current provider, google-beta 7.43.0 -- re-verified). TWO REAL ROOT CAUSES found and fixed for why Model Armor was never actually invoked: (1) IAM was granted to the wrong Service Extensions service agent -- assumed to be service-{our project number}@gcp-sa-dep.iam.gserviceaccount.com, but direct REST evidence (querying the gateway resource's own agentGatewayCard.serviceExtensionsServiceAccount field) proved the real principal is a different, Google-internal tenant project. Fixed via Terraform referencing the gateway's own computed attribute. (2) A stale warm container (&gt;40min uptime) was bypassing gateway interception entirely for the custom MCP host. AFTER both fixes, Model Armor invocation is genuinely proven live (real ext_proc calls, grpcStatus=OK, serviceExtensionInfo populated) on both the custom MCP and GKE Remote MCP paths -- confirmed via gcloud logging read against networkservices.googleapis.com/Gateway. REMAINING GAP, now understood precisely: RESPONSE_BODY never fires as an ext_proc event for MCP tools/call responses on either path. Google's own Model Armor + Agent Gateway integration docs state 'Streamable HTTP/SSE for MCP' is allowed without sanitization -- our custom MCP's own code proves it uses exactly this transport (mcp/server.py:442, transport='streamable-http'). Two independent malicious payloads (prompt-injection, and Google's own guaranteed-detection Safe Browsing URL) both passed through unblocked on this path, tested on both the custom MCP AND Google's own GKE Remote MCP path (corroborating, not primary, evidence -- GKE Remote MCP's internal transport is not published by Google). DECISION (explicit, 2026-09-05): accepted as a proven, documented Google platform limitation -- not a code defect, not silently reclassified as a lesser Phase 1.1 item. Phase 1 OpenSpec acceptance criterion #203 recorded as PARTIAL -- ACCEPTED PLATFORM LIMITATION. Floor-setting mechanism (row 21/122) continues providing real inspect-only detection as a disclosed, compensating control -- NOT equivalent to CONTENT_AUTHZ blocking. NEXT: a Google Cloud support case will be filed as a non-blocking follow-up (confirmation + roadmap ask) -- Phase 1 completion does not wait for a response. Full evidence: PHASE1_EVIDENCE_LOG.md and GitHub issue #203 comment, feat/phase-1-release branch.</t>
+          <t>UPDATED 2026-09-05. Investigated end to end on feat/phase-1-release. Fixed the original gating bug this row describes, plus corrected agent_gateway.tf's stale comment (the gateway-side CONTENT_AUTHZ extension DOES exist on the current provider, google-beta 7.43.0 -- re-verified). TWO REAL ROOT CAUSES found and fixed for why Model Armor was never actually invoked: (1) IAM was granted to the wrong Service Extensions service agent -- assumed to be service-{our project number}@gcp-sa-dep.iam.gserviceaccount.com, but direct REST evidence (querying the gateway resource's own agentGatewayCard.serviceExtensionsServiceAccount field) proved the real principal is a different, Google-internal tenant project. Fixed via Terraform referencing the gateway's own computed attribute. (2) A stale warm container (&gt;40min uptime) was bypassing gateway interception entirely for the custom MCP host. AFTER both fixes, Model Armor invocation is genuinely proven live (real ext_proc calls, grpcStatus=OK, serviceExtensionInfo populated) on both the custom MCP and GKE Remote MCP paths -- confirmed via gcloud logging read against networkservices.googleapis.com/Gateway. REMAINING GAP, now understood precisely: RESPONSE_BODY never fires as an ext_proc event for MCP tools/call responses on either path. Google's own Model Armor + Agent Gateway integration docs state 'Streamable HTTP/SSE for MCP' is allowed without sanitization -- our custom MCP's own code proves it uses exactly this transport (mcp/server.py:442, transport='streamable-http'). Two independent malicious payloads (prompt-injection, and Google's own guaranteed-detection Safe Browsing URL) both passed through unblocked on this path, tested on both the custom MCP AND Google's own GKE Remote MCP path (corroborating, not primary, evidence -- GKE Remote MCP's internal transport is not published by Google). DECISION (explicit, 2026-09-05): accepted as a proven, documented Google platform limitation -- not a code defect, not silently reclassified as a lesser Phase 1.1 item. Phase 1 OpenSpec acceptance criterion #203 recorded as PARTIAL -- ACCEPTED PLATFORM LIMITATION. Floor-setting mechanism (row 21/122) continues providing real inspect-only detection as a disclosed, compensating control -- NOT equivalent to CONTENT_AUTHZ blocking. NEXT: a Google Cloud support case will be filed as a non-blocking follow-up (confirmation + roadmap ask) -- Phase 1 completion does not wait for a response. Full evidence: PHASE1_EVIDENCE_LOG.md and GitHub issue #203 comment, feat/phase-1-release branch. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z, commit dc6f022 + 5f2d136): shipped a compensating control for the RESPONSE_BODY gap on the custom MCP path specifically -- mcp/response_guard.py, a FastMCP on_call_tool middleware that calls Model Armor's sanitize_model_response directly against the sre_agent_response template, closing the gap CONTENT_AUTHZ cannot for this one MCP source. CI green (mcp-pytest, pytest, plan all pass). Deployed via CI terraform-apply (run 34054067651; first attempt failed on a real, understood GCP Cloud Monitoring metric-propagation 404 -- 'could not find metric, try again in up to 10 min' -- re-ran the same job with no code change once propagated, succeeded). Live-proven on the merged deployment: normal investigation run_20260906_192633_snql (status=done, selected_mcp=k8s_mcp); malicious-response run_20260906_192834_yoqw -- 2x real BLOCK, MCP log 'ModelArmorResponseGuard BLOCKED tool response tool=describe_pod_detail', Model Armor sanitize_operations log MODEL_ARMOR_SANITIZATION_VERDICT_BLOCK / malicious_uris MATCH_FOUND on the exact test URL at byte offset 310-361; agent responded truthfully (status=done, error=null, confidence=0.0, no fabricated RCA). Guard fails OPEN on a Model Armor API error -- deliberate, disclosed availability tradeoff (read-only architecture bounds the worst case to corrupted evidence/RCA text; every RCA already requires human review regardless; fail-closed would take the investigation tool down during real incidents over an unrelated dependency outage). Loud alerting added to back that decision: new google_logging_metric + google_monitoring_alert_policy 'sre_agent/mcp_model_armor_fail_open' (verified beforehand that NO existing alert matched this event -- filters on textPayload, not severity, since Cloud Run's default stdout capture for this service's plain Python logging shows an empty severity field even on WARNING/ERROR lines, confirmed live). Terraform drift-check after deploy: 0 add, 1 change (reasoning-engine source_archive -- known local-vs-CI build non-determinism, unrelated to this change), 0 destroy. NOT closing this row/#203 -- response-side inspection for GKE Remote MCP remains an accepted platform limitation (row unchanged), and the Google Cloud support case this row's own prior note commits to filing has still not been filed. Full evidence in GitHub issue #203 comment and PHASE1_EVIDENCE_LOG.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs(tracker): re-verify rows 121/165 unchanged, note #86/#246/#202 have no dedicated tracker row
</commit_message>
<xml_diff>
--- a/docs/management/PROJECT_TRACKER.xlsx
+++ b/docs/management/PROJECT_TRACKER.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet name="Project Tracker" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Phase Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Reference" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="External Dependencies" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Completed" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="In Progress" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Not Started" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Blocked" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Deferred" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Tracker" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Phase Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reference" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="External Dependencies" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Completed" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="In Progress" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not Started" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deferred" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
 </workbook>
@@ -268,14 +268,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:lstStyle/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:lstStyle xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:r>
               <a:t>Tasks by Status</a:t>
             </a:r>
@@ -295,7 +295,7 @@
             <v>Series 1</v>
           </tx>
           <spPr>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -330,7 +330,7 @@
         <axPos val="b"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -356,7 +356,7 @@
         <axPos val="l"/>
         <majorGridlines>
           <spPr>
-            <a:ln w="9525">
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
               <a:solidFill>
                 <a:srgbClr val="CCCCCC"/>
               </a:solidFill>
@@ -375,7 +375,7 @@
     <dispBlanksAs val="gap"/>
   </chart>
   <spPr>
-    <a:ln w="9525">
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
       <a:solidFill>
         <a:srgbClr val="D9D9D9"/>
       </a:solidFill>
@@ -386,7 +386,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <twoCellAnchor>
     <from>
       <col>6</col>
@@ -406,9 +406,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -6377,7 +6377,7 @@
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Final production review. | UPDATE 2026-09-05: REQUEST_AUTHZ staleness/bypass test completed -- revoked the agent identity's roles/iap.egressor binding on an already-warm (&gt;5h) connection, retried immediately: denied within 2.8s, gateway log shows authzPolicyInfo.result=DENIED on the very first egress attempt, zero stale-enforcement window. Restored, confirmed access works again, confirmed zero Terraform drift. Verdict: PASS, no bypass, confirmed against official Google docs (authz extensions invoke live at the request-headers stage, no cache). See PHASE1_EVIDENCE_LOG.md. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z): the REQUEST_AUTHZ staleness/bypass test above (2026-09-05) was investigation-only -- authz_fail_open was still true by default. This PR makes the fix durable: iac/agent/variables.tf's authz_fail_open default changed true -&gt; false, merged, deployed via CI (run 34054067651), confirmed live via `terraform state show` (google_network_services_authz_extension.iap[0].fail_open = false). Not independently re-tested post-merge beyond confirming the live value (the underlying revoke/retry/no-bypass behavior was already proven 2026-09-05 against the same mechanism). NOT marking this row Completed -- 'Agent Gateway security validation' / 'Final Agent Gateway production validation' covers more than this one fix (CONTENT_AUTHZ response-side gap, row 165/#203, remains open).</t>
+          <t>Final production review. | UPDATE 2026-09-05: REQUEST_AUTHZ staleness/bypass test completed -- revoked the agent identity's roles/iap.egressor binding on an already-warm (&gt;5h) connection, retried immediately: denied within 2.8s, gateway log shows authzPolicyInfo.result=DENIED on the very first egress attempt, zero stale-enforcement window. Restored, confirmed access works again, confirmed zero Terraform drift. Verdict: PASS, no bypass, confirmed against official Google docs (authz extensions invoke live at the request-headers stage, no cache). See PHASE1_EVIDENCE_LOG.md. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z): the REQUEST_AUTHZ staleness/bypass test above (2026-09-05) was investigation-only -- authz_fail_open was still true by default. This PR makes the fix durable: iac/agent/variables.tf's authz_fail_open default changed true -&gt; false, merged, deployed via CI (run 34054067651), confirmed live via `terraform state show` (google_network_services_authz_extension.iap[0].fail_open = false). Not independently re-tested post-merge beyond confirming the live value (the underlying revoke/retry/no-bypass behavior was already proven 2026-09-05 against the same mechanism). NOT marking this row Completed -- 'Agent Gateway security validation' / 'Final Agent Gateway production validation' covers more than this one fix (CONTENT_AUTHZ response-side gap, row 165/#203, remains open). | UPDATE 2026-09-07 (Phase 1 Final Readiness review, verify-only): re-confirmed live -- google_network_services_authz_extension.iap[0].fail_open = false, unchanged since PR #249. No new work this session on this row; #246 (separate cluster-scoped tool-argument bug, no dedicated tracker row) fixed and live-tested on review branch phase1-final-readiness-review, see GitHub issue #246.</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>UPDATED 2026-09-05. Investigated end to end on feat/phase-1-release. Fixed the original gating bug this row describes, plus corrected agent_gateway.tf's stale comment (the gateway-side CONTENT_AUTHZ extension DOES exist on the current provider, google-beta 7.43.0 -- re-verified). TWO REAL ROOT CAUSES found and fixed for why Model Armor was never actually invoked: (1) IAM was granted to the wrong Service Extensions service agent -- assumed to be service-{our project number}@gcp-sa-dep.iam.gserviceaccount.com, but direct REST evidence (querying the gateway resource's own agentGatewayCard.serviceExtensionsServiceAccount field) proved the real principal is a different, Google-internal tenant project. Fixed via Terraform referencing the gateway's own computed attribute. (2) A stale warm container (&gt;40min uptime) was bypassing gateway interception entirely for the custom MCP host. AFTER both fixes, Model Armor invocation is genuinely proven live (real ext_proc calls, grpcStatus=OK, serviceExtensionInfo populated) on both the custom MCP and GKE Remote MCP paths -- confirmed via gcloud logging read against networkservices.googleapis.com/Gateway. REMAINING GAP, now understood precisely: RESPONSE_BODY never fires as an ext_proc event for MCP tools/call responses on either path. Google's own Model Armor + Agent Gateway integration docs state 'Streamable HTTP/SSE for MCP' is allowed without sanitization -- our custom MCP's own code proves it uses exactly this transport (mcp/server.py:442, transport='streamable-http'). Two independent malicious payloads (prompt-injection, and Google's own guaranteed-detection Safe Browsing URL) both passed through unblocked on this path, tested on both the custom MCP AND Google's own GKE Remote MCP path (corroborating, not primary, evidence -- GKE Remote MCP's internal transport is not published by Google). DECISION (explicit, 2026-09-05): accepted as a proven, documented Google platform limitation -- not a code defect, not silently reclassified as a lesser Phase 1.1 item. Phase 1 OpenSpec acceptance criterion #203 recorded as PARTIAL -- ACCEPTED PLATFORM LIMITATION. Floor-setting mechanism (row 21/122) continues providing real inspect-only detection as a disclosed, compensating control -- NOT equivalent to CONTENT_AUTHZ blocking. NEXT: a Google Cloud support case will be filed as a non-blocking follow-up (confirmation + roadmap ask) -- Phase 1 completion does not wait for a response. Full evidence: PHASE1_EVIDENCE_LOG.md and GitHub issue #203 comment, feat/phase-1-release branch. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z, commit dc6f022 + 5f2d136): shipped a compensating control for the RESPONSE_BODY gap on the custom MCP path specifically -- mcp/response_guard.py, a FastMCP on_call_tool middleware that calls Model Armor's sanitize_model_response directly against the sre_agent_response template, closing the gap CONTENT_AUTHZ cannot for this one MCP source. CI green (mcp-pytest, pytest, plan all pass). Deployed via CI terraform-apply (run 34054067651; first attempt failed on a real, understood GCP Cloud Monitoring metric-propagation 404 -- 'could not find metric, try again in up to 10 min' -- re-ran the same job with no code change once propagated, succeeded). Live-proven on the merged deployment: normal investigation run_20260906_192633_snql (status=done, selected_mcp=k8s_mcp); malicious-response run_20260906_192834_yoqw -- 2x real BLOCK, MCP log 'ModelArmorResponseGuard BLOCKED tool response tool=describe_pod_detail', Model Armor sanitize_operations log MODEL_ARMOR_SANITIZATION_VERDICT_BLOCK / malicious_uris MATCH_FOUND on the exact test URL at byte offset 310-361; agent responded truthfully (status=done, error=null, confidence=0.0, no fabricated RCA). Guard fails OPEN on a Model Armor API error -- deliberate, disclosed availability tradeoff (read-only architecture bounds the worst case to corrupted evidence/RCA text; every RCA already requires human review regardless; fail-closed would take the investigation tool down during real incidents over an unrelated dependency outage). Loud alerting added to back that decision: new google_logging_metric + google_monitoring_alert_policy 'sre_agent/mcp_model_armor_fail_open' (verified beforehand that NO existing alert matched this event -- filters on textPayload, not severity, since Cloud Run's default stdout capture for this service's plain Python logging shows an empty severity field even on WARNING/ERROR lines, confirmed live). Terraform drift-check after deploy: 0 add, 1 change (reasoning-engine source_archive -- known local-vs-CI build non-determinism, unrelated to this change), 0 destroy. NOT closing this row/#203 -- response-side inspection for GKE Remote MCP remains an accepted platform limitation (row unchanged), and the Google Cloud support case this row's own prior note commits to filing has still not been filed. Full evidence in GitHub issue #203 comment and PHASE1_EVIDENCE_LOG.md.</t>
+          <t>UPDATED 2026-09-05. Investigated end to end on feat/phase-1-release. Fixed the original gating bug this row describes, plus corrected agent_gateway.tf's stale comment (the gateway-side CONTENT_AUTHZ extension DOES exist on the current provider, google-beta 7.43.0 -- re-verified). TWO REAL ROOT CAUSES found and fixed for why Model Armor was never actually invoked: (1) IAM was granted to the wrong Service Extensions service agent -- assumed to be service-{our project number}@gcp-sa-dep.iam.gserviceaccount.com, but direct REST evidence (querying the gateway resource's own agentGatewayCard.serviceExtensionsServiceAccount field) proved the real principal is a different, Google-internal tenant project. Fixed via Terraform referencing the gateway's own computed attribute. (2) A stale warm container (&gt;40min uptime) was bypassing gateway interception entirely for the custom MCP host. AFTER both fixes, Model Armor invocation is genuinely proven live (real ext_proc calls, grpcStatus=OK, serviceExtensionInfo populated) on both the custom MCP and GKE Remote MCP paths -- confirmed via gcloud logging read against networkservices.googleapis.com/Gateway. REMAINING GAP, now understood precisely: RESPONSE_BODY never fires as an ext_proc event for MCP tools/call responses on either path. Google's own Model Armor + Agent Gateway integration docs state 'Streamable HTTP/SSE for MCP' is allowed without sanitization -- our custom MCP's own code proves it uses exactly this transport (mcp/server.py:442, transport='streamable-http'). Two independent malicious payloads (prompt-injection, and Google's own guaranteed-detection Safe Browsing URL) both passed through unblocked on this path, tested on both the custom MCP AND Google's own GKE Remote MCP path (corroborating, not primary, evidence -- GKE Remote MCP's internal transport is not published by Google). DECISION (explicit, 2026-09-05): accepted as a proven, documented Google platform limitation -- not a code defect, not silently reclassified as a lesser Phase 1.1 item. Phase 1 OpenSpec acceptance criterion #203 recorded as PARTIAL -- ACCEPTED PLATFORM LIMITATION. Floor-setting mechanism (row 21/122) continues providing real inspect-only detection as a disclosed, compensating control -- NOT equivalent to CONTENT_AUTHZ blocking. NEXT: a Google Cloud support case will be filed as a non-blocking follow-up (confirmation + roadmap ask) -- Phase 1 completion does not wait for a response. Full evidence: PHASE1_EVIDENCE_LOG.md and GitHub issue #203 comment, feat/phase-1-release branch. | UPDATE 2026-09-06 (PR #249, merged 2026-09-06T19:10:49Z, commit dc6f022 + 5f2d136): shipped a compensating control for the RESPONSE_BODY gap on the custom MCP path specifically -- mcp/response_guard.py, a FastMCP on_call_tool middleware that calls Model Armor's sanitize_model_response directly against the sre_agent_response template, closing the gap CONTENT_AUTHZ cannot for this one MCP source. CI green (mcp-pytest, pytest, plan all pass). Deployed via CI terraform-apply (run 34054067651; first attempt failed on a real, understood GCP Cloud Monitoring metric-propagation 404 -- 'could not find metric, try again in up to 10 min' -- re-ran the same job with no code change once propagated, succeeded). Live-proven on the merged deployment: normal investigation run_20260906_192633_snql (status=done, selected_mcp=k8s_mcp); malicious-response run_20260906_192834_yoqw -- 2x real BLOCK, MCP log 'ModelArmorResponseGuard BLOCKED tool response tool=describe_pod_detail', Model Armor sanitize_operations log MODEL_ARMOR_SANITIZATION_VERDICT_BLOCK / malicious_uris MATCH_FOUND on the exact test URL at byte offset 310-361; agent responded truthfully (status=done, error=null, confidence=0.0, no fabricated RCA). Guard fails OPEN on a Model Armor API error -- deliberate, disclosed availability tradeoff (read-only architecture bounds the worst case to corrupted evidence/RCA text; every RCA already requires human review regardless; fail-closed would take the investigation tool down during real incidents over an unrelated dependency outage). Loud alerting added to back that decision: new google_logging_metric + google_monitoring_alert_policy 'sre_agent/mcp_model_armor_fail_open' (verified beforehand that NO existing alert matched this event -- filters on textPayload, not severity, since Cloud Run's default stdout capture for this service's plain Python logging shows an empty severity field even on WARNING/ERROR lines, confirmed live). Terraform drift-check after deploy: 0 add, 1 change (reasoning-engine source_archive -- known local-vs-CI build non-determinism, unrelated to this change), 0 destroy. NOT closing this row/#203 -- response-side inspection for GKE Remote MCP remains an accepted platform limitation (row unchanged), and the Google Cloud support case this row's own prior note commits to filing has still not been filed. Full evidence in GitHub issue #203 comment and PHASE1_EVIDENCE_LOG.md. | UPDATE 2026-09-07 (Phase 1 Final Readiness review, verify-only): re-confirmed live -- response guard still deployed and actively blocking (real BLOCKED event observed 2026-09-06T19:28Z, unrelated prior traffic), floor settings still HIGH+INSPECT_ONLY, RESPONSE_BODY gap still present (3-day log spot-check, zero events) -- unchanged platform limitation, not re-litigated. Google Support case still a draft, not filed. No new work this session on this row.</t>
         </is>
       </c>
     </row>

</xml_diff>